<commit_message>
working with two voltmeters
</commit_message>
<xml_diff>
--- a/AMP_0dB_result.xlsx
+++ b/AMP_0dB_result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrew\Desktop\боц8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0932931-1CF0-454F-A4D5-4F09A858A824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E54E4FE8-AD24-4256-BB2B-C4DC6D1F8699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1485" yWindow="2280" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1224,28 +1224,28 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="M6" s="2">
-        <v>4.9653760999999998E-2</v>
+        <v>4.9646522999999998E-2</v>
       </c>
       <c r="N6" s="2">
-        <v>4.9321233999999999E-2</v>
+        <v>4.9421634999999998E-2</v>
       </c>
       <c r="O6" s="2">
-        <v>4.9180500000000002E-2</v>
+        <v>4.9365847999999997E-2</v>
       </c>
       <c r="P6" s="2">
-        <v>4.9507253000000001E-2</v>
+        <v>4.9648929000000001E-2</v>
       </c>
       <c r="Q6" s="2">
-        <v>4.9128740999999997E-2</v>
+        <v>4.9479544E-2</v>
       </c>
       <c r="R6" s="2">
-        <v>4.9335215000000002E-2</v>
+        <v>4.9539614000000003E-2</v>
       </c>
       <c r="S6" s="2">
-        <v>4.9280303999999997E-2</v>
+        <v>4.9420538999999999E-2</v>
       </c>
       <c r="T6" s="2">
-        <v>4.9383799999999999E-2</v>
+        <v>4.9484028999999999E-2</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -1285,28 +1285,28 @@
         <v>0.01</v>
       </c>
       <c r="M7" s="2">
-        <v>9.9257796999999995E-2</v>
+        <v>9.9198118000000002E-2</v>
       </c>
       <c r="N7" s="2">
-        <v>9.8648049000000002E-2</v>
+        <v>9.8798311999999999E-2</v>
       </c>
       <c r="O7" s="2">
-        <v>9.8337635000000007E-2</v>
+        <v>9.8645738999999996E-2</v>
       </c>
       <c r="P7" s="2">
-        <v>9.8979570000000003E-2</v>
+        <v>9.9203199000000006E-2</v>
       </c>
       <c r="Q7" s="2">
-        <v>9.8292999000000006E-2</v>
+        <v>9.8892412999999998E-2</v>
       </c>
       <c r="R7" s="2">
-        <v>9.8645248000000005E-2</v>
+        <v>9.8972641E-2</v>
       </c>
       <c r="S7" s="2">
-        <v>9.8550877999999995E-2</v>
+        <v>9.8797508000000006E-2</v>
       </c>
       <c r="T7" s="2">
-        <v>9.8765119999999998E-2</v>
+        <v>9.8897360000000004E-2</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -1315,59 +1315,59 @@
       </c>
       <c r="B8" s="3">
         <f t="shared" si="1"/>
-        <v>4.9653760999999998E-2</v>
+        <v>4.9646522999999998E-2</v>
       </c>
       <c r="C8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9321233999999999E-2</v>
+        <v>4.9421634999999998E-2</v>
       </c>
       <c r="D8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9180500000000002E-2</v>
+        <v>4.9365847999999997E-2</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9507253000000001E-2</v>
+        <v>4.9648929000000001E-2</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9128740999999997E-2</v>
+        <v>4.9479544E-2</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9335215000000002E-2</v>
+        <v>4.9539614000000003E-2</v>
       </c>
       <c r="H8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9280303999999997E-2</v>
+        <v>4.9420538999999999E-2</v>
       </c>
       <c r="I8" s="3">
         <f t="shared" si="0"/>
-        <v>4.9383799999999999E-2</v>
+        <v>4.9484028999999999E-2</v>
       </c>
       <c r="M8" s="2">
-        <v>0.13851919800000001</v>
+        <v>0.13837860499999999</v>
       </c>
       <c r="N8" s="2">
-        <v>0.13771715800000001</v>
+        <v>0.13785354799999999</v>
       </c>
       <c r="O8" s="2">
-        <v>0.13728334</v>
+        <v>0.13761501000000001</v>
       </c>
       <c r="P8" s="2">
-        <v>0.138157591</v>
+        <v>0.13838911100000001</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.13725939400000001</v>
+        <v>0.137969434</v>
       </c>
       <c r="R8" s="2">
-        <v>0.137703821</v>
+        <v>0.13806226799999999</v>
       </c>
       <c r="S8" s="2">
-        <v>0.13758574400000001</v>
+        <v>0.13784992700000001</v>
       </c>
       <c r="T8" s="2">
-        <v>0.137886748</v>
+        <v>0.137978509</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
@@ -1376,59 +1376,59 @@
       </c>
       <c r="B9" s="3">
         <f t="shared" si="1"/>
-        <v>9.9257796999999995E-2</v>
+        <v>9.9198118000000002E-2</v>
       </c>
       <c r="C9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8648049000000002E-2</v>
+        <v>9.8798311999999999E-2</v>
       </c>
       <c r="D9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8337635000000007E-2</v>
+        <v>9.8645738999999996E-2</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8979570000000003E-2</v>
+        <v>9.9203199000000006E-2</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8292999000000006E-2</v>
+        <v>9.8892412999999998E-2</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8645248000000005E-2</v>
+        <v>9.8972641E-2</v>
       </c>
       <c r="H9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8550877999999995E-2</v>
+        <v>9.8797508000000006E-2</v>
       </c>
       <c r="I9" s="3">
         <f t="shared" si="0"/>
-        <v>9.8765119999999998E-2</v>
+        <v>9.8897360000000004E-2</v>
       </c>
       <c r="M9" s="2">
-        <v>1.4327904499999999E-4</v>
+        <v>1.4062308800000001E-4</v>
       </c>
       <c r="N9" s="2">
-        <v>1.2032071400000001E-4</v>
+        <v>1.30052067E-4</v>
       </c>
       <c r="O9" s="2">
-        <v>9.2437462000000007E-5</v>
+        <v>1.5196319099999999E-4</v>
       </c>
       <c r="P9" s="2">
-        <v>1.0819365E-4</v>
+        <v>1.3572778000000001E-4</v>
       </c>
       <c r="Q9" s="2">
-        <v>1.1232378899999999E-4</v>
+        <v>1.471617E-4</v>
       </c>
       <c r="R9" s="2">
-        <v>1.1767627400000001E-4</v>
+        <v>1.3898707400000001E-4</v>
       </c>
       <c r="S9" s="2">
-        <v>1.27992273E-4</v>
+        <v>1.5942650499999999E-4</v>
       </c>
       <c r="T9" s="2">
-        <v>1.0090452300000001E-4</v>
+        <v>1.49539352E-4</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
@@ -1437,85 +1437,85 @@
       </c>
       <c r="B10" s="3">
         <f t="shared" si="1"/>
-        <v>0.13851919800000001</v>
+        <v>0.13837860499999999</v>
       </c>
       <c r="C10" s="3">
         <f t="shared" si="0"/>
-        <v>0.13771715800000001</v>
+        <v>0.13785354799999999</v>
       </c>
       <c r="D10" s="3">
         <f t="shared" si="0"/>
-        <v>0.13728334</v>
+        <v>0.13761501000000001</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="0"/>
-        <v>0.138157591</v>
+        <v>0.13838911100000001</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>0.13725939400000001</v>
+        <v>0.137969434</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="0"/>
-        <v>0.137703821</v>
+        <v>0.13806226799999999</v>
       </c>
       <c r="H10" s="3">
         <f t="shared" si="0"/>
-        <v>0.13758574400000001</v>
+        <v>0.13784992700000001</v>
       </c>
       <c r="I10" s="3">
         <f t="shared" si="0"/>
-        <v>0.137886748</v>
+        <v>0.137978509</v>
       </c>
       <c r="M10" s="2">
-        <v>3.4339481500000001E-4</v>
+        <v>4.1626876899999998E-4</v>
       </c>
       <c r="N10" s="2">
-        <v>3.3408618799999999E-4</v>
+        <v>4.1352081500000001E-4</v>
       </c>
       <c r="O10" s="2">
-        <v>3.4013367300000003E-4</v>
+        <v>4.0043404400000001E-4</v>
       </c>
       <c r="P10" s="2">
-        <v>3.5267355299999998E-4</v>
+        <v>4.1544897199999998E-4</v>
       </c>
       <c r="Q10" s="2">
-        <v>3.4568223099999999E-4</v>
+        <v>4.0115061000000002E-4</v>
       </c>
       <c r="R10" s="2">
-        <v>3.2404588999999999E-4</v>
+        <v>4.2745214899999999E-4</v>
       </c>
       <c r="S10" s="2">
-        <v>3.6018722999999999E-4</v>
+        <v>3.88639251E-4</v>
       </c>
       <c r="T10" s="2">
-        <v>3.4185842399999999E-4</v>
+        <v>4.0060566999999998E-4</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="M11" s="2">
-        <v>7.5840967500000005E-4</v>
+        <v>8.3247816699999998E-4</v>
       </c>
       <c r="N11" s="2">
-        <v>7.3902169200000002E-4</v>
+        <v>8.2078797300000003E-4</v>
       </c>
       <c r="O11" s="2">
-        <v>7.4906478400000003E-4</v>
+        <v>8.1655860399999997E-4</v>
       </c>
       <c r="P11" s="2">
-        <v>7.6447025600000001E-4</v>
+        <v>8.3343271400000002E-4</v>
       </c>
       <c r="Q11" s="2">
-        <v>7.5305870300000004E-4</v>
+        <v>8.1965647400000004E-4</v>
       </c>
       <c r="R11" s="2">
-        <v>7.5939384999999999E-4</v>
+        <v>8.2085363100000005E-4</v>
       </c>
       <c r="S11" s="2">
-        <v>7.5143342800000005E-4</v>
+        <v>8.1815233000000003E-4</v>
       </c>
       <c r="T11" s="2">
-        <v>7.5859099200000001E-4</v>
+        <v>8.1713689699999998E-4</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
@@ -1531,28 +1531,28 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="M12" s="2">
-        <v>4.7142360000000001E-3</v>
+        <v>4.6998500000000002E-3</v>
       </c>
       <c r="N12" s="2">
-        <v>4.6898809999999999E-3</v>
+        <v>4.6635950000000004E-3</v>
       </c>
       <c r="O12" s="2">
-        <v>4.6807419999999999E-3</v>
+        <v>4.6729520000000002E-3</v>
       </c>
       <c r="P12" s="2">
-        <v>4.6991519999999998E-3</v>
+        <v>4.7036530000000003E-3</v>
       </c>
       <c r="Q12" s="2">
-        <v>4.7008359999999999E-3</v>
+        <v>4.6629150000000001E-3</v>
       </c>
       <c r="R12" s="2">
-        <v>4.6836409999999997E-3</v>
+        <v>4.6867339999999997E-3</v>
       </c>
       <c r="S12" s="2">
-        <v>4.6854089999999998E-3</v>
+        <v>4.6987130000000002E-3</v>
       </c>
       <c r="T12" s="2">
-        <v>4.692641E-3</v>
+        <v>4.694475E-3</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
@@ -1584,28 +1584,28 @@
         <v>8</v>
       </c>
       <c r="M13" s="2">
-        <v>9.6913989999999998E-3</v>
+        <v>9.6651280000000003E-3</v>
       </c>
       <c r="N13" s="2">
-        <v>9.6087350000000002E-3</v>
+        <v>9.6069729999999996E-3</v>
       </c>
       <c r="O13" s="2">
-        <v>9.5906029999999996E-3</v>
+        <v>9.6211400000000002E-3</v>
       </c>
       <c r="P13" s="2">
-        <v>9.6345509999999999E-3</v>
+        <v>9.6860820000000004E-3</v>
       </c>
       <c r="Q13" s="2">
-        <v>9.6105119999999999E-3</v>
+        <v>9.6272830000000004E-3</v>
       </c>
       <c r="R13" s="2">
-        <v>9.6409660000000008E-3</v>
+        <v>9.6334179999999995E-3</v>
       </c>
       <c r="S13" s="2">
-        <v>9.6443950000000001E-3</v>
+        <v>9.6606560000000001E-3</v>
       </c>
       <c r="T13" s="2">
-        <v>9.6232020000000008E-3</v>
+        <v>9.6279409999999992E-3</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
@@ -1614,59 +1614,59 @@
       </c>
       <c r="B14" s="3">
         <f>M9*1000000</f>
-        <v>143.279045</v>
+        <v>140.62308800000002</v>
       </c>
       <c r="C14" s="3">
         <f t="shared" ref="C14:I14" si="2">N9*1000000</f>
-        <v>120.32071400000001</v>
+        <v>130.05206699999999</v>
       </c>
       <c r="D14" s="3">
         <f t="shared" si="2"/>
-        <v>92.437462000000011</v>
+        <v>151.96319099999999</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" si="2"/>
-        <v>108.19365000000001</v>
+        <v>135.72778000000002</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" si="2"/>
-        <v>112.32378899999999</v>
+        <v>147.1617</v>
       </c>
       <c r="G14" s="3">
         <f t="shared" si="2"/>
-        <v>117.67627400000001</v>
+        <v>138.98707400000001</v>
       </c>
       <c r="H14" s="3">
         <f t="shared" si="2"/>
-        <v>127.992273</v>
+        <v>159.42650499999999</v>
       </c>
       <c r="I14" s="3">
         <f t="shared" si="2"/>
-        <v>100.90452300000001</v>
+        <v>149.53935200000001</v>
       </c>
       <c r="M14" s="2">
-        <v>4.8971523000000003E-2</v>
+        <v>4.9167178999999998E-2</v>
       </c>
       <c r="N14" s="2">
-        <v>4.8679106E-2</v>
+        <v>4.8775021000000002E-2</v>
       </c>
       <c r="O14" s="2">
-        <v>4.8527832999999999E-2</v>
+        <v>4.8803959000000001E-2</v>
       </c>
       <c r="P14" s="2">
-        <v>4.8900235E-2</v>
+        <v>4.9220745000000003E-2</v>
       </c>
       <c r="Q14" s="2">
-        <v>4.8685428000000003E-2</v>
+        <v>4.8881341000000002E-2</v>
       </c>
       <c r="R14" s="2">
-        <v>4.8609554999999999E-2</v>
+        <v>4.8878860000000003E-2</v>
       </c>
       <c r="S14" s="2">
-        <v>4.8649116999999999E-2</v>
+        <v>4.8939864999999999E-2</v>
       </c>
       <c r="T14" s="2">
-        <v>4.8746556000000003E-2</v>
+        <v>4.8893467000000003E-2</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
@@ -1675,59 +1675,59 @@
       </c>
       <c r="B15" s="3">
         <f>M10*1000000</f>
-        <v>343.39481499999999</v>
+        <v>416.26876899999996</v>
       </c>
       <c r="C15" s="3">
         <f t="shared" ref="C15:C20" si="3">N10*1000000</f>
-        <v>334.08618799999999</v>
+        <v>413.52081500000003</v>
       </c>
       <c r="D15" s="3">
         <f t="shared" ref="D15:D20" si="4">O10*1000000</f>
-        <v>340.13367300000004</v>
+        <v>400.43404400000003</v>
       </c>
       <c r="E15" s="3">
         <f t="shared" ref="E15:E20" si="5">P10*1000000</f>
-        <v>352.67355299999997</v>
+        <v>415.44897199999997</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" ref="F15:F20" si="6">Q10*1000000</f>
-        <v>345.682231</v>
+        <v>401.15061000000003</v>
       </c>
       <c r="G15" s="3">
         <f t="shared" ref="G15:G20" si="7">R10*1000000</f>
-        <v>324.04588999999999</v>
+        <v>427.45214899999996</v>
       </c>
       <c r="H15" s="3">
         <f t="shared" ref="H15:H20" si="8">S10*1000000</f>
-        <v>360.18723</v>
+        <v>388.639251</v>
       </c>
       <c r="I15" s="3">
         <f t="shared" ref="I15:I20" si="9">T10*1000000</f>
-        <v>341.85842400000001</v>
+        <v>400.60566999999998</v>
       </c>
       <c r="M15" s="2">
-        <v>9.8080135999999998E-2</v>
+        <v>9.8323076999999995E-2</v>
       </c>
       <c r="N15" s="2">
-        <v>9.7578891000000001E-2</v>
+        <v>9.7828506999999995E-2</v>
       </c>
       <c r="O15" s="2">
-        <v>9.7522057999999995E-2</v>
+        <v>9.7695677999999994E-2</v>
       </c>
       <c r="P15" s="2">
-        <v>9.7994179000000001E-2</v>
+        <v>9.8404527000000006E-2</v>
       </c>
       <c r="Q15" s="2">
-        <v>9.7385845999999998E-2</v>
+        <v>9.7643710999999994E-2</v>
       </c>
       <c r="R15" s="2">
-        <v>9.7453265999999997E-2</v>
+        <v>9.8148114999999994E-2</v>
       </c>
       <c r="S15" s="2">
-        <v>9.7543694E-2</v>
+        <v>9.7977623E-2</v>
       </c>
       <c r="T15" s="2">
-        <v>9.7655423000000005E-2</v>
+        <v>9.7819231000000006E-2</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
@@ -1736,59 +1736,59 @@
       </c>
       <c r="B16" s="3">
         <f t="shared" ref="B16:B20" si="10">M11*1000000</f>
-        <v>758.40967499999999</v>
+        <v>832.47816699999998</v>
       </c>
       <c r="C16" s="3">
         <f>N11*1000000</f>
-        <v>739.02169200000003</v>
+        <v>820.78797300000008</v>
       </c>
       <c r="D16" s="3">
         <f t="shared" si="4"/>
-        <v>749.06478400000003</v>
+        <v>816.55860399999995</v>
       </c>
       <c r="E16" s="3">
         <f t="shared" si="5"/>
-        <v>764.47025600000006</v>
+        <v>833.43271400000003</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" si="6"/>
-        <v>753.05870300000004</v>
+        <v>819.656474</v>
       </c>
       <c r="G16" s="3">
         <f t="shared" si="7"/>
-        <v>759.39385000000004</v>
+        <v>820.85363100000006</v>
       </c>
       <c r="H16" s="3">
         <f t="shared" si="8"/>
-        <v>751.43342800000005</v>
+        <v>818.15233000000001</v>
       </c>
       <c r="I16" s="3">
         <f t="shared" si="9"/>
-        <v>758.59099200000003</v>
+        <v>817.13689699999998</v>
       </c>
       <c r="M16" s="2">
-        <v>0.13710075599999999</v>
+        <v>0.13762374199999999</v>
       </c>
       <c r="N16" s="2">
-        <v>0.13633622200000001</v>
+        <v>0.136526078</v>
       </c>
       <c r="O16" s="2">
-        <v>0.13645607200000001</v>
+        <v>0.13652241200000001</v>
       </c>
       <c r="P16" s="2">
-        <v>0.137001291</v>
+        <v>0.13746804000000001</v>
       </c>
       <c r="Q16" s="2">
-        <v>0.13603758799999999</v>
+        <v>0.136401415</v>
       </c>
       <c r="R16" s="2">
-        <v>0.136684373</v>
+        <v>0.13687759599999999</v>
       </c>
       <c r="S16" s="2">
-        <v>0.13648934700000001</v>
+        <v>0.13686870000000001</v>
       </c>
       <c r="T16" s="2">
-        <v>0.136221856</v>
+        <v>0.13662481300000001</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
@@ -1797,35 +1797,35 @@
       </c>
       <c r="B17" s="3">
         <f t="shared" si="10"/>
-        <v>4714.2359999999999</v>
+        <v>4699.8500000000004</v>
       </c>
       <c r="C17" s="3">
         <f t="shared" si="3"/>
-        <v>4689.8810000000003</v>
+        <v>4663.5950000000003</v>
       </c>
       <c r="D17" s="3">
         <f t="shared" si="4"/>
-        <v>4680.7420000000002</v>
+        <v>4672.9520000000002</v>
       </c>
       <c r="E17" s="3">
         <f t="shared" si="5"/>
-        <v>4699.152</v>
+        <v>4703.6530000000002</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" si="6"/>
-        <v>4700.8360000000002</v>
+        <v>4662.915</v>
       </c>
       <c r="G17" s="3">
         <f t="shared" si="7"/>
-        <v>4683.6409999999996</v>
+        <v>4686.7339999999995</v>
       </c>
       <c r="H17" s="3">
         <f t="shared" si="8"/>
-        <v>4685.4089999999997</v>
+        <v>4698.7130000000006</v>
       </c>
       <c r="I17" s="3">
         <f t="shared" si="9"/>
-        <v>4692.6409999999996</v>
+        <v>4694.4750000000004</v>
       </c>
       <c r="M17" s="2">
         <v>9.9999997000000003E-5</v>
@@ -1858,35 +1858,35 @@
       </c>
       <c r="B18" s="3">
         <f t="shared" si="10"/>
-        <v>9691.3989999999994</v>
+        <v>9665.1280000000006</v>
       </c>
       <c r="C18" s="3">
         <f t="shared" si="3"/>
-        <v>9608.7350000000006</v>
+        <v>9606.973</v>
       </c>
       <c r="D18" s="3">
         <f t="shared" si="4"/>
-        <v>9590.6029999999992</v>
+        <v>9621.14</v>
       </c>
       <c r="E18" s="3">
         <f t="shared" si="5"/>
-        <v>9634.5509999999995</v>
+        <v>9686.0820000000003</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" si="6"/>
-        <v>9610.5120000000006</v>
+        <v>9627.2830000000013</v>
       </c>
       <c r="G18" s="3">
         <f t="shared" si="7"/>
-        <v>9640.9660000000003</v>
+        <v>9633.4179999999997</v>
       </c>
       <c r="H18" s="3">
         <f t="shared" si="8"/>
-        <v>9644.3950000000004</v>
+        <v>9660.6560000000009</v>
       </c>
       <c r="I18" s="3">
         <f t="shared" si="9"/>
-        <v>9623.2020000000011</v>
+        <v>9627.9409999999989</v>
       </c>
       <c r="M18" s="2">
         <v>5.0000002400000002E-4</v>
@@ -1919,35 +1919,35 @@
       </c>
       <c r="B19" s="3">
         <f t="shared" si="10"/>
-        <v>48971.523000000001</v>
+        <v>49167.178999999996</v>
       </c>
       <c r="C19" s="3">
         <f t="shared" si="3"/>
-        <v>48679.106</v>
+        <v>48775.021000000001</v>
       </c>
       <c r="D19" s="3">
         <f t="shared" si="4"/>
-        <v>48527.832999999999</v>
+        <v>48803.959000000003</v>
       </c>
       <c r="E19" s="3">
         <f t="shared" si="5"/>
-        <v>48900.235000000001</v>
+        <v>49220.745000000003</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" si="6"/>
-        <v>48685.428</v>
+        <v>48881.341</v>
       </c>
       <c r="G19" s="3">
         <f t="shared" si="7"/>
-        <v>48609.555</v>
+        <v>48878.86</v>
       </c>
       <c r="H19" s="3">
         <f t="shared" si="8"/>
-        <v>48649.116999999998</v>
+        <v>48939.864999999998</v>
       </c>
       <c r="I19" s="3">
         <f t="shared" si="9"/>
-        <v>48746.556000000004</v>
+        <v>48893.467000000004</v>
       </c>
       <c r="M19" s="2">
         <v>1E-3</v>
@@ -1980,35 +1980,35 @@
       </c>
       <c r="B20" s="3">
         <f t="shared" si="10"/>
-        <v>98080.135999999999</v>
+        <v>98323.07699999999</v>
       </c>
       <c r="C20" s="3">
         <f t="shared" si="3"/>
-        <v>97578.891000000003</v>
+        <v>97828.506999999998</v>
       </c>
       <c r="D20" s="3">
         <f t="shared" si="4"/>
-        <v>97522.05799999999</v>
+        <v>97695.678</v>
       </c>
       <c r="E20" s="3">
         <f t="shared" si="5"/>
-        <v>97994.179000000004</v>
+        <v>98404.527000000002</v>
       </c>
       <c r="F20" s="3">
         <f t="shared" si="6"/>
-        <v>97385.846000000005</v>
+        <v>97643.710999999996</v>
       </c>
       <c r="G20" s="3">
         <f t="shared" si="7"/>
-        <v>97453.266000000003</v>
+        <v>98148.114999999991</v>
       </c>
       <c r="H20" s="3">
         <f t="shared" si="8"/>
-        <v>97543.694000000003</v>
+        <v>97977.623000000007</v>
       </c>
       <c r="I20" s="3">
         <f t="shared" si="9"/>
-        <v>97655.42300000001</v>
+        <v>97819.231</v>
       </c>
       <c r="M20" s="2">
         <v>5.0000000000000001E-3</v>
@@ -2041,35 +2041,35 @@
       </c>
       <c r="B21" s="3">
         <f t="shared" ref="B21:I21" si="11">M16*1000000</f>
-        <v>137100.75599999999</v>
+        <v>137623.742</v>
       </c>
       <c r="C21" s="3">
         <f t="shared" si="11"/>
-        <v>136336.22200000001</v>
+        <v>136526.07800000001</v>
       </c>
       <c r="D21" s="3">
         <f t="shared" si="11"/>
-        <v>136456.07200000001</v>
+        <v>136522.41200000001</v>
       </c>
       <c r="E21" s="3">
         <f t="shared" si="11"/>
-        <v>137001.291</v>
+        <v>137468.04</v>
       </c>
       <c r="F21" s="3">
         <f t="shared" si="11"/>
-        <v>136037.58799999999</v>
+        <v>136401.41500000001</v>
       </c>
       <c r="G21" s="3">
         <f t="shared" si="11"/>
-        <v>136684.37299999999</v>
+        <v>136877.59599999999</v>
       </c>
       <c r="H21" s="3">
         <f t="shared" si="11"/>
-        <v>136489.34700000001</v>
+        <v>136868.70000000001</v>
       </c>
       <c r="I21" s="3">
         <f t="shared" si="11"/>
-        <v>136221.856</v>
+        <v>136624.81300000002</v>
       </c>
       <c r="M21" s="2">
         <v>0.01</v>
@@ -2098,28 +2098,28 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="M22" s="2">
-        <v>4.9657185E-2</v>
+        <v>4.9648944E-2</v>
       </c>
       <c r="N22" s="2">
-        <v>4.9322214000000003E-2</v>
+        <v>4.9422151999999997E-2</v>
       </c>
       <c r="O22" s="2">
-        <v>4.9180210000000002E-2</v>
+        <v>4.9366750000000001E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>4.9510393E-2</v>
+        <v>4.9650144E-2</v>
       </c>
       <c r="Q22" s="2">
-        <v>4.9127109000000002E-2</v>
+        <v>4.9479201E-2</v>
       </c>
       <c r="R22" s="2">
-        <v>4.9333009999999997E-2</v>
+        <v>4.9541768E-2</v>
       </c>
       <c r="S22" s="2">
-        <v>4.9280927000000002E-2</v>
+        <v>4.9420486999999999E-2</v>
       </c>
       <c r="T22" s="2">
-        <v>4.9382417999999997E-2</v>
+        <v>4.9485080000000001E-2</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
@@ -2135,28 +2135,28 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="M23" s="2">
-        <v>9.9257380000000006E-2</v>
+        <v>9.9197707999999996E-2</v>
       </c>
       <c r="N23" s="2">
-        <v>9.8652601000000006E-2</v>
+        <v>9.8801247999999994E-2</v>
       </c>
       <c r="O23" s="2">
-        <v>9.8352060000000005E-2</v>
+        <v>9.8655022999999994E-2</v>
       </c>
       <c r="P23" s="2">
-        <v>9.8990790999999995E-2</v>
+        <v>9.9213228000000001E-2</v>
       </c>
       <c r="Q23" s="2">
-        <v>9.8291390000000006E-2</v>
+        <v>9.8898418000000002E-2</v>
       </c>
       <c r="R23" s="2">
-        <v>9.8654150999999995E-2</v>
+        <v>9.8980001999999997E-2</v>
       </c>
       <c r="S23" s="2">
-        <v>9.8553099000000005E-2</v>
+        <v>9.8801970000000003E-2</v>
       </c>
       <c r="T23" s="2">
-        <v>9.8756610999999994E-2</v>
+        <v>9.8901956999999999E-2</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
@@ -2188,28 +2188,28 @@
         <v>8</v>
       </c>
       <c r="M24" s="2">
-        <v>0.13853174400000001</v>
+        <v>0.13836736999999999</v>
       </c>
       <c r="N24" s="2">
-        <v>0.13772116600000001</v>
+        <v>0.13784755800000001</v>
       </c>
       <c r="O24" s="2">
-        <v>0.13727302799999999</v>
+        <v>0.137628257</v>
       </c>
       <c r="P24" s="2">
-        <v>0.13815058799999999</v>
+        <v>0.13840269999999999</v>
       </c>
       <c r="Q24" s="2">
-        <v>0.137254819</v>
+        <v>0.13797804699999999</v>
       </c>
       <c r="R24" s="2">
-        <v>0.13769927600000001</v>
+        <v>0.13806575500000001</v>
       </c>
       <c r="S24" s="2">
-        <v>0.137584448</v>
+        <v>0.13786093899999999</v>
       </c>
       <c r="T24" s="2">
-        <v>0.137880057</v>
+        <v>0.13798896999999999</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
@@ -2218,59 +2218,59 @@
       </c>
       <c r="B25" s="1">
         <f>B14-B3</f>
-        <v>143.27894500000301</v>
+        <v>140.62298800000303</v>
       </c>
       <c r="C25" s="1">
         <f t="shared" ref="C25:I25" si="12">C14-C3</f>
-        <v>120.320614000003</v>
+        <v>130.051967000003</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" si="12"/>
-        <v>92.437362000003006</v>
+        <v>151.963091000003</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" si="12"/>
-        <v>108.193550000003</v>
+        <v>135.72768000000303</v>
       </c>
       <c r="F25" s="1">
         <f t="shared" si="12"/>
-        <v>112.32368900000299</v>
+        <v>147.16160000000301</v>
       </c>
       <c r="G25" s="1">
         <f t="shared" si="12"/>
-        <v>117.676174000003</v>
+        <v>138.98697400000302</v>
       </c>
       <c r="H25" s="1">
         <f t="shared" si="12"/>
-        <v>127.99217300000299</v>
+        <v>159.426405000003</v>
       </c>
       <c r="I25" s="1">
         <f t="shared" si="12"/>
-        <v>100.90442300000301</v>
+        <v>149.53925200000302</v>
       </c>
       <c r="M25" s="2">
-        <v>1.5249993899999999E-4</v>
+        <v>1.21754252E-4</v>
       </c>
       <c r="N25" s="2">
-        <v>1.4064095700000001E-4</v>
+        <v>1.20793382E-4</v>
       </c>
       <c r="O25" s="2">
-        <v>1.4630715299999999E-4</v>
+        <v>1.22003032E-4</v>
       </c>
       <c r="P25" s="2">
-        <v>1.4388884299999999E-4</v>
+        <v>1.2682679499999999E-4</v>
       </c>
       <c r="Q25" s="2">
-        <v>1.5208304100000001E-4</v>
+        <v>1.2481863100000001E-4</v>
       </c>
       <c r="R25" s="2">
-        <v>1.56417998E-4</v>
+        <v>1.26072264E-4</v>
       </c>
       <c r="S25" s="2">
-        <v>1.3809143299999999E-4</v>
+        <v>1.2147550299999999E-4</v>
       </c>
       <c r="T25" s="2">
-        <v>1.4500779800000001E-4</v>
+        <v>1.1922544900000001E-4</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
@@ -2279,59 +2279,59 @@
       </c>
       <c r="B26" s="1">
         <f t="shared" ref="B26:I26" si="13">B15-B4</f>
-        <v>343.39431499997602</v>
+        <v>416.26826899997599</v>
       </c>
       <c r="C26" s="1">
         <f t="shared" si="13"/>
-        <v>334.08568799997602</v>
+        <v>413.52031499997605</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" si="13"/>
-        <v>340.13317299997607</v>
+        <v>400.43354399997605</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" si="13"/>
-        <v>352.67305299997599</v>
+        <v>415.44847199997599</v>
       </c>
       <c r="F26" s="1">
         <f t="shared" si="13"/>
-        <v>345.68173099997603</v>
+        <v>401.15010999997605</v>
       </c>
       <c r="G26" s="1">
         <f t="shared" si="13"/>
-        <v>324.04538999997601</v>
+        <v>427.45164899997599</v>
       </c>
       <c r="H26" s="1">
         <f t="shared" si="13"/>
-        <v>360.18672999997602</v>
+        <v>388.63875099997603</v>
       </c>
       <c r="I26" s="1">
         <f t="shared" si="13"/>
-        <v>341.85792399997604</v>
+        <v>400.605169999976</v>
       </c>
       <c r="M26" s="2">
-        <v>4.8140744899999999E-4</v>
+        <v>4.7682001600000002E-4</v>
       </c>
       <c r="N26" s="2">
-        <v>4.8673912500000002E-4</v>
+        <v>4.7615493500000001E-4</v>
       </c>
       <c r="O26" s="2">
-        <v>4.9431267000000004E-4</v>
+        <v>4.7731155099999998E-4</v>
       </c>
       <c r="P26" s="2">
-        <v>4.8781884800000002E-4</v>
+        <v>4.7420134099999999E-4</v>
       </c>
       <c r="Q26" s="2">
-        <v>4.8768019800000001E-4</v>
+        <v>4.7280560799999998E-4</v>
       </c>
       <c r="R26" s="2">
-        <v>4.8726514800000002E-4</v>
+        <v>4.7671387400000001E-4</v>
       </c>
       <c r="S26" s="2">
-        <v>4.8279372300000001E-4</v>
+        <v>4.7571072399999999E-4</v>
       </c>
       <c r="T26" s="2">
-        <v>4.8004451699999999E-4</v>
+        <v>4.6621434699999997E-4</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
@@ -2340,59 +2340,59 @@
       </c>
       <c r="B27" s="1">
         <f t="shared" ref="B27:I27" si="14">B16-B5</f>
-        <v>758.40867500000002</v>
+        <v>832.47716700000001</v>
       </c>
       <c r="C27" s="1">
         <f t="shared" si="14"/>
-        <v>739.02069200000005</v>
+        <v>820.7869730000001</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" si="14"/>
-        <v>749.06378400000006</v>
+        <v>816.55760399999997</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" si="14"/>
-        <v>764.46925600000009</v>
+        <v>833.43171400000006</v>
       </c>
       <c r="F27" s="1">
         <f t="shared" si="14"/>
-        <v>753.05770300000006</v>
+        <v>819.65547400000003</v>
       </c>
       <c r="G27" s="1">
         <f t="shared" si="14"/>
-        <v>759.39285000000007</v>
+        <v>820.85263100000009</v>
       </c>
       <c r="H27" s="1">
         <f t="shared" si="14"/>
-        <v>751.43242800000007</v>
+        <v>818.15133000000003</v>
       </c>
       <c r="I27" s="1">
         <f t="shared" si="14"/>
-        <v>758.58999200000005</v>
+        <v>817.135897</v>
       </c>
       <c r="M27" s="2">
-        <v>9.8831742099999989E-4</v>
+        <v>9.7306759599999999E-4</v>
       </c>
       <c r="N27" s="2">
-        <v>9.7154261299999998E-4</v>
+        <v>9.6003862599999996E-4</v>
       </c>
       <c r="O27" s="2">
-        <v>9.8478992000000003E-4</v>
+        <v>9.7187486199999998E-4</v>
       </c>
       <c r="P27" s="2">
-        <v>9.7897730300000011E-4</v>
+        <v>9.7793142800000005E-4</v>
       </c>
       <c r="Q27" s="2">
-        <v>9.8658294900000006E-4</v>
+        <v>9.5944979699999998E-4</v>
       </c>
       <c r="R27" s="2">
-        <v>9.9140463900000003E-4</v>
+        <v>9.7522459700000001E-4</v>
       </c>
       <c r="S27" s="2">
-        <v>9.6484430800000004E-4</v>
+        <v>9.7100000099999996E-4</v>
       </c>
       <c r="T27" s="2">
-        <v>9.6528546399999996E-4</v>
+        <v>9.72567359E-4</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
@@ -2401,59 +2401,59 @@
       </c>
       <c r="B28" s="1">
         <f t="shared" ref="B28:I28" si="15">B17-B6</f>
-        <v>4714.2309999999998</v>
+        <v>4699.8450000000003</v>
       </c>
       <c r="C28" s="1">
         <f t="shared" si="15"/>
-        <v>4689.8760000000002</v>
+        <v>4663.59</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" si="15"/>
-        <v>4680.7370000000001</v>
+        <v>4672.9470000000001</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" si="15"/>
-        <v>4699.1469999999999</v>
+        <v>4703.6480000000001</v>
       </c>
       <c r="F28" s="1">
         <f t="shared" si="15"/>
-        <v>4700.8310000000001</v>
+        <v>4662.91</v>
       </c>
       <c r="G28" s="1">
         <f t="shared" si="15"/>
-        <v>4683.6359999999995</v>
+        <v>4686.7289999999994</v>
       </c>
       <c r="H28" s="1">
         <f t="shared" si="15"/>
-        <v>4685.4039999999995</v>
+        <v>4698.7080000000005</v>
       </c>
       <c r="I28" s="1">
         <f t="shared" si="15"/>
-        <v>4692.6359999999995</v>
+        <v>4694.47</v>
       </c>
       <c r="M28" s="2">
-        <v>4.945044E-3</v>
+        <v>4.9523889999999997E-3</v>
       </c>
       <c r="N28" s="2">
-        <v>4.9320550000000003E-3</v>
+        <v>4.9363870000000004E-3</v>
       </c>
       <c r="O28" s="2">
-        <v>4.9637290000000001E-3</v>
+        <v>4.9431659999999997E-3</v>
       </c>
       <c r="P28" s="2">
-        <v>4.9496030000000003E-3</v>
+        <v>4.9300539999999997E-3</v>
       </c>
       <c r="Q28" s="2">
-        <v>4.9678450000000002E-3</v>
+        <v>4.9443910000000002E-3</v>
       </c>
       <c r="R28" s="2">
-        <v>4.9425449999999996E-3</v>
+        <v>4.9511690000000001E-3</v>
       </c>
       <c r="S28" s="2">
-        <v>4.9452649999999999E-3</v>
+        <v>4.9516289999999999E-3</v>
       </c>
       <c r="T28" s="2">
-        <v>4.9295800000000002E-3</v>
+        <v>4.9385399999999999E-3</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
@@ -2462,59 +2462,59 @@
       </c>
       <c r="B29" s="1">
         <f t="shared" ref="B29:I29" si="16">B18-B7</f>
-        <v>9691.3889999999992</v>
+        <v>9665.1180000000004</v>
       </c>
       <c r="C29" s="1">
         <f t="shared" si="16"/>
-        <v>9608.7250000000004</v>
+        <v>9606.9629999999997</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" si="16"/>
-        <v>9590.5929999999989</v>
+        <v>9621.1299999999992</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" si="16"/>
-        <v>9634.5409999999993</v>
+        <v>9686.0720000000001</v>
       </c>
       <c r="F29" s="1">
         <f t="shared" si="16"/>
-        <v>9610.5020000000004</v>
+        <v>9627.273000000001</v>
       </c>
       <c r="G29" s="1">
         <f t="shared" si="16"/>
-        <v>9640.9560000000001</v>
+        <v>9633.4079999999994</v>
       </c>
       <c r="H29" s="1">
         <f t="shared" si="16"/>
-        <v>9644.3850000000002</v>
+        <v>9660.6460000000006</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="16"/>
-        <v>9623.1920000000009</v>
+        <v>9627.9309999999987</v>
       </c>
       <c r="M29" s="2">
-        <v>9.9152419999999995E-3</v>
+        <v>9.9412860000000006E-3</v>
       </c>
       <c r="N29" s="2">
-        <v>9.9014270000000008E-3</v>
+        <v>9.8977070000000004E-3</v>
       </c>
       <c r="O29" s="2">
-        <v>9.9509590000000005E-3</v>
+        <v>9.9254010000000004E-3</v>
       </c>
       <c r="P29" s="2">
-        <v>9.9225609999999999E-3</v>
+        <v>9.9105949999999995E-3</v>
       </c>
       <c r="Q29" s="2">
-        <v>9.9393869999999992E-3</v>
+        <v>9.9115539999999995E-3</v>
       </c>
       <c r="R29" s="2">
-        <v>9.9205419999999992E-3</v>
+        <v>9.9514819999999993E-3</v>
       </c>
       <c r="S29" s="2">
-        <v>9.8962040000000005E-3</v>
+        <v>9.9236340000000006E-3</v>
       </c>
       <c r="T29" s="2">
-        <v>9.8879759999999997E-3</v>
+        <v>9.9391700000000006E-3</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
@@ -2523,59 +2523,59 @@
       </c>
       <c r="B30" s="1">
         <f t="shared" ref="B30:I30" si="17">B19-B8</f>
-        <v>48971.473346239</v>
+        <v>49167.129353476994</v>
       </c>
       <c r="C30" s="1">
         <f t="shared" si="17"/>
-        <v>48679.056678765999</v>
+        <v>48774.971578365003</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" si="17"/>
-        <v>48527.7838195</v>
+        <v>48803.909634152005</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" si="17"/>
-        <v>48900.185492746998</v>
+        <v>49220.695351071001</v>
       </c>
       <c r="F30" s="1">
         <f t="shared" si="17"/>
-        <v>48685.378871259003</v>
+        <v>48881.291520455998</v>
       </c>
       <c r="G30" s="1">
         <f t="shared" si="17"/>
-        <v>48609.505664785</v>
+        <v>48878.810460385997</v>
       </c>
       <c r="H30" s="1">
         <f t="shared" si="17"/>
-        <v>48649.067719695995</v>
+        <v>48939.815579460999</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="17"/>
-        <v>48746.506616200008</v>
+        <v>48893.417515971007</v>
       </c>
       <c r="M30" s="2">
-        <v>4.9462076000000001E-2</v>
+        <v>4.9533903999999997E-2</v>
       </c>
       <c r="N30" s="2">
-        <v>4.9399658999999999E-2</v>
+        <v>4.9345898999999999E-2</v>
       </c>
       <c r="O30" s="2">
-        <v>4.9613386000000002E-2</v>
+        <v>4.9606129999999998E-2</v>
       </c>
       <c r="P30" s="2">
-        <v>4.950073E-2</v>
+        <v>4.9413449999999998E-2</v>
       </c>
       <c r="Q30" s="2">
-        <v>4.9618807000000001E-2</v>
+        <v>4.9467183999999997E-2</v>
       </c>
       <c r="R30" s="2">
-        <v>4.9608263999999999E-2</v>
+        <v>4.9669549E-2</v>
       </c>
       <c r="S30" s="2">
-        <v>4.947878E-2</v>
+        <v>4.9623596999999998E-2</v>
       </c>
       <c r="T30" s="2">
-        <v>4.9246727999999997E-2</v>
+        <v>4.9498691999999997E-2</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
@@ -2584,59 +2584,59 @@
       </c>
       <c r="B31" s="1">
         <f t="shared" ref="B31:I31" si="18">B20-B9</f>
-        <v>98080.036742202996</v>
+        <v>98322.977801881992</v>
       </c>
       <c r="C31" s="1">
         <f t="shared" si="18"/>
-        <v>97578.792351951008</v>
+        <v>97828.408201687998</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" si="18"/>
-        <v>97521.959662364985</v>
+        <v>97695.579354261004</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" si="18"/>
-        <v>97994.080020430003</v>
+        <v>98404.427796800999</v>
       </c>
       <c r="F31" s="1">
         <f t="shared" si="18"/>
-        <v>97385.747707001006</v>
+        <v>97643.612107586989</v>
       </c>
       <c r="G31" s="1">
         <f t="shared" si="18"/>
-        <v>97453.167354752004</v>
+        <v>98148.016027358986</v>
       </c>
       <c r="H31" s="1">
         <f t="shared" si="18"/>
-        <v>97543.595449122004</v>
+        <v>97977.524202492001</v>
       </c>
       <c r="I31" s="1">
         <f t="shared" si="18"/>
-        <v>97655.324234880012</v>
+        <v>97819.132102639996</v>
       </c>
       <c r="M31" s="2">
-        <v>9.8821133000000005E-2</v>
+        <v>9.8989137000000005E-2</v>
       </c>
       <c r="N31" s="2">
-        <v>9.8632857000000004E-2</v>
+        <v>9.8584621999999997E-2</v>
       </c>
       <c r="O31" s="2">
-        <v>9.9286689999999997E-2</v>
+        <v>9.9155969999999996E-2</v>
       </c>
       <c r="P31" s="2">
-        <v>9.8927698999999994E-2</v>
+        <v>9.8913893000000003E-2</v>
       </c>
       <c r="Q31" s="2">
-        <v>9.8993323999999994E-2</v>
+        <v>9.8725349000000004E-2</v>
       </c>
       <c r="R31" s="2">
-        <v>9.9263869000000005E-2</v>
+        <v>9.9280454000000004E-2</v>
       </c>
       <c r="S31" s="2">
-        <v>9.8892674E-2</v>
+        <v>9.9077529999999997E-2</v>
       </c>
       <c r="T31" s="2">
-        <v>9.8489434000000001E-2</v>
+        <v>9.8777868000000005E-2</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
@@ -2645,59 +2645,59 @@
       </c>
       <c r="B32" s="1">
         <f t="shared" ref="B32:I32" si="19">B21-B10</f>
-        <v>137100.617480802</v>
+        <v>137623.60362139498</v>
       </c>
       <c r="C32" s="1">
         <f t="shared" si="19"/>
-        <v>136336.084282842</v>
+        <v>136525.94014645202</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" si="19"/>
-        <v>136455.93471666001</v>
+        <v>136522.27438499001</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" si="19"/>
-        <v>137001.15284240901</v>
+        <v>137467.90161088901</v>
       </c>
       <c r="F32" s="1">
         <f t="shared" si="19"/>
-        <v>136037.450740606</v>
+        <v>136401.27703056601</v>
       </c>
       <c r="G32" s="1">
         <f t="shared" si="19"/>
-        <v>136684.23529617899</v>
+        <v>136877.45793773199</v>
       </c>
       <c r="H32" s="1">
         <f t="shared" si="19"/>
-        <v>136489.20941425601</v>
+        <v>136868.562150073</v>
       </c>
       <c r="I32" s="1">
         <f t="shared" si="19"/>
-        <v>136221.71811325199</v>
+        <v>136624.67502149101</v>
       </c>
       <c r="M32" s="2">
-        <v>0.115692213</v>
+        <v>0.114988878</v>
       </c>
       <c r="N32" s="2">
-        <v>0.11365082899999999</v>
+        <v>0.11341332599999999</v>
       </c>
       <c r="O32" s="2">
-        <v>0.11513762900000001</v>
+        <v>0.115133464</v>
       </c>
       <c r="P32" s="2">
-        <v>0.11497713599999999</v>
+        <v>0.114165224</v>
       </c>
       <c r="Q32" s="2">
-        <v>0.112903349</v>
+        <v>0.114818394</v>
       </c>
       <c r="R32" s="2">
-        <v>0.114548489</v>
+        <v>0.115638897</v>
       </c>
       <c r="S32" s="2">
-        <v>0.11361903700000001</v>
+        <v>0.114336312</v>
       </c>
       <c r="T32" s="2">
-        <v>0.114151902</v>
+        <v>0.114496373</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
@@ -2940,28 +2940,28 @@
         <v>5.0000002400000002E-4</v>
       </c>
       <c r="M38" s="2">
-        <v>4.9655095000000003E-2</v>
+        <v>4.9650811000000003E-2</v>
       </c>
       <c r="N38" s="2">
-        <v>4.9324519999999997E-2</v>
+        <v>4.9422219000000003E-2</v>
       </c>
       <c r="O38" s="2">
-        <v>4.9180791000000001E-2</v>
+        <v>4.9367290000000001E-2</v>
       </c>
       <c r="P38" s="2">
-        <v>4.9508496999999999E-2</v>
+        <v>4.9646094000000002E-2</v>
       </c>
       <c r="Q38" s="2">
-        <v>4.9131345E-2</v>
+        <v>4.9480746999999999E-2</v>
       </c>
       <c r="R38" s="2">
-        <v>4.9340144000000002E-2</v>
+        <v>4.9538441000000003E-2</v>
       </c>
       <c r="S38" s="2">
-        <v>4.9281432999999999E-2</v>
+        <v>4.9419998999999999E-2</v>
       </c>
       <c r="T38" s="2">
-        <v>4.9382750000000003E-2</v>
+        <v>4.9482878000000001E-2</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.25">
@@ -3001,28 +3001,28 @@
         <v>1E-3</v>
       </c>
       <c r="M39" s="2">
-        <v>9.9262929999999999E-2</v>
+        <v>9.9202491000000004E-2</v>
       </c>
       <c r="N39" s="2">
-        <v>9.8648741999999998E-2</v>
+        <v>9.8805428000000001E-2</v>
       </c>
       <c r="O39" s="2">
-        <v>9.8343431999999995E-2</v>
+        <v>9.8655857E-2</v>
       </c>
       <c r="P39" s="2">
-        <v>9.8990038000000002E-2</v>
+        <v>9.9210665000000003E-2</v>
       </c>
       <c r="Q39" s="2">
-        <v>9.8295055000000006E-2</v>
+        <v>9.8896242999999995E-2</v>
       </c>
       <c r="R39" s="2">
-        <v>9.8657139000000005E-2</v>
+        <v>9.8978109999999994E-2</v>
       </c>
       <c r="S39" s="2">
-        <v>9.8554007999999999E-2</v>
+        <v>9.8800674000000005E-2</v>
       </c>
       <c r="T39" s="2">
-        <v>9.8760411000000006E-2</v>
+        <v>9.8902008999999999E-2</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
@@ -3062,28 +3062,28 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="M40" s="2">
-        <v>0.13853786900000001</v>
+        <v>0.138369307</v>
       </c>
       <c r="N40" s="2">
-        <v>0.13773238700000001</v>
+        <v>0.137844458</v>
       </c>
       <c r="O40" s="2">
-        <v>0.13728112000000001</v>
+        <v>0.137627363</v>
       </c>
       <c r="P40" s="2">
-        <v>0.138173938</v>
+        <v>0.138406157</v>
       </c>
       <c r="Q40" s="2">
-        <v>0.13726683000000001</v>
+        <v>0.137964159</v>
       </c>
       <c r="R40" s="2">
-        <v>0.137702301</v>
+        <v>0.13806495099999999</v>
       </c>
       <c r="S40" s="2">
-        <v>0.137587458</v>
+        <v>0.13785430800000001</v>
       </c>
       <c r="T40" s="2">
-        <v>0.13789103899999999</v>
+        <v>0.13798032700000001</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
@@ -3123,28 +3123,28 @@
         <v>0.01</v>
       </c>
       <c r="M41" s="2">
-        <v>3.18033097E-4</v>
+        <v>4.2472046300000001E-4</v>
       </c>
       <c r="N41" s="2">
-        <v>3.0771232600000002E-4</v>
+        <v>4.2089994499999999E-4</v>
       </c>
       <c r="O41" s="2">
-        <v>3.4788099599999999E-4</v>
+        <v>3.9224186899999998E-4</v>
       </c>
       <c r="P41" s="2">
-        <v>3.62225634E-4</v>
+        <v>4.07368847E-4</v>
       </c>
       <c r="Q41" s="2">
-        <v>3.3692212300000002E-4</v>
+        <v>4.3490721100000003E-4</v>
       </c>
       <c r="R41" s="2">
-        <v>3.1576535500000001E-4</v>
+        <v>4.0809460900000002E-4</v>
       </c>
       <c r="S41" s="2">
-        <v>3.4917215799999999E-4</v>
+        <v>4.1191294399999998E-4</v>
       </c>
       <c r="T41" s="2">
-        <v>3.3369485799999998E-4</v>
+        <v>4.3565040699999999E-4</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.25">
@@ -3153,59 +3153,59 @@
       </c>
       <c r="B42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9657185E-2</v>
+        <v>4.9648944E-2</v>
       </c>
       <c r="C42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9322214000000003E-2</v>
+        <v>4.9422151999999997E-2</v>
       </c>
       <c r="D42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9180210000000002E-2</v>
+        <v>4.9366750000000001E-2</v>
       </c>
       <c r="E42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9510393E-2</v>
+        <v>4.9650144E-2</v>
       </c>
       <c r="F42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9127109000000002E-2</v>
+        <v>4.9479201E-2</v>
       </c>
       <c r="G42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9333009999999997E-2</v>
+        <v>4.9541768E-2</v>
       </c>
       <c r="H42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9280927000000002E-2</v>
+        <v>4.9420486999999999E-2</v>
       </c>
       <c r="I42" s="3">
         <f t="shared" si="20"/>
-        <v>4.9382417999999997E-2</v>
+        <v>4.9485080000000001E-2</v>
       </c>
       <c r="M42" s="2">
-        <v>2.2108869999999999E-3</v>
+        <v>2.171086E-3</v>
       </c>
       <c r="N42" s="2">
-        <v>2.1889119999999999E-3</v>
+        <v>2.14504E-3</v>
       </c>
       <c r="O42" s="2">
-        <v>2.198729E-3</v>
+        <v>2.1632349999999999E-3</v>
       </c>
       <c r="P42" s="2">
-        <v>2.19418E-3</v>
+        <v>2.1721140000000002E-3</v>
       </c>
       <c r="Q42" s="2">
-        <v>2.1981679999999999E-3</v>
+        <v>2.15226E-3</v>
       </c>
       <c r="R42" s="2">
-        <v>2.1744939999999999E-3</v>
+        <v>2.1547409999999999E-3</v>
       </c>
       <c r="S42" s="2">
-        <v>2.1768400000000002E-3</v>
+        <v>2.1567940000000001E-3</v>
       </c>
       <c r="T42" s="2">
-        <v>2.2001949999999998E-3</v>
+        <v>2.1687529999999998E-3</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
@@ -3214,59 +3214,59 @@
       </c>
       <c r="B43" s="3">
         <f t="shared" si="20"/>
-        <v>9.9257380000000006E-2</v>
+        <v>9.9197707999999996E-2</v>
       </c>
       <c r="C43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8652601000000006E-2</v>
+        <v>9.8801247999999994E-2</v>
       </c>
       <c r="D43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8352060000000005E-2</v>
+        <v>9.8655022999999994E-2</v>
       </c>
       <c r="E43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8990790999999995E-2</v>
+        <v>9.9213228000000001E-2</v>
       </c>
       <c r="F43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8291390000000006E-2</v>
+        <v>9.8898418000000002E-2</v>
       </c>
       <c r="G43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8654150999999995E-2</v>
+        <v>9.8980001999999997E-2</v>
       </c>
       <c r="H43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8553099000000005E-2</v>
+        <v>9.8801970000000003E-2</v>
       </c>
       <c r="I43" s="3">
         <f t="shared" si="20"/>
-        <v>9.8756610999999994E-2</v>
+        <v>9.8901956999999999E-2</v>
       </c>
       <c r="M43" s="2">
-        <v>4.7174890000000001E-3</v>
+        <v>4.6861059999999998E-3</v>
       </c>
       <c r="N43" s="2">
-        <v>4.7002049999999998E-3</v>
+        <v>4.6889039999999998E-3</v>
       </c>
       <c r="O43" s="2">
-        <v>4.6898829999999997E-3</v>
+        <v>4.6756929999999999E-3</v>
       </c>
       <c r="P43" s="2">
-        <v>4.6962530000000001E-3</v>
+        <v>4.70382E-3</v>
       </c>
       <c r="Q43" s="2">
-        <v>4.6702990000000002E-3</v>
+        <v>4.6825670000000003E-3</v>
       </c>
       <c r="R43" s="2">
-        <v>4.6772960000000001E-3</v>
+        <v>4.6702640000000004E-3</v>
       </c>
       <c r="S43" s="2">
-        <v>4.6846580000000004E-3</v>
+        <v>4.683792E-3</v>
       </c>
       <c r="T43" s="2">
-        <v>4.7044230000000001E-3</v>
+        <v>4.6806590000000002E-3</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
@@ -3275,85 +3275,85 @@
       </c>
       <c r="B44" s="3">
         <f t="shared" si="20"/>
-        <v>0.13853174400000001</v>
+        <v>0.13836736999999999</v>
       </c>
       <c r="C44" s="3">
         <f t="shared" si="20"/>
-        <v>0.13772116600000001</v>
+        <v>0.13784755800000001</v>
       </c>
       <c r="D44" s="3">
         <f t="shared" si="20"/>
-        <v>0.13727302799999999</v>
+        <v>0.137628257</v>
       </c>
       <c r="E44" s="3">
         <f t="shared" si="20"/>
-        <v>0.13815058799999999</v>
+        <v>0.13840269999999999</v>
       </c>
       <c r="F44" s="3">
         <f t="shared" si="20"/>
-        <v>0.137254819</v>
+        <v>0.13797804699999999</v>
       </c>
       <c r="G44" s="3">
         <f t="shared" si="20"/>
-        <v>0.13769927600000001</v>
+        <v>0.13806575500000001</v>
       </c>
       <c r="H44" s="3">
         <f t="shared" si="20"/>
-        <v>0.137584448</v>
+        <v>0.13786093899999999</v>
       </c>
       <c r="I44" s="3">
         <f t="shared" si="20"/>
-        <v>0.137880057</v>
+        <v>0.13798896999999999</v>
       </c>
       <c r="M44" s="2">
-        <v>2.4677900999999999E-2</v>
+        <v>2.4681225000000001E-2</v>
       </c>
       <c r="N44" s="2">
-        <v>2.4517210000000001E-2</v>
+        <v>2.4502705999999999E-2</v>
       </c>
       <c r="O44" s="2">
-        <v>2.4482248000000002E-2</v>
+        <v>2.4452728999999999E-2</v>
       </c>
       <c r="P44" s="2">
-        <v>2.4537674999999998E-2</v>
+        <v>2.4673168999999998E-2</v>
       </c>
       <c r="Q44" s="2">
-        <v>2.4481973000000001E-2</v>
+        <v>2.4532681000000001E-2</v>
       </c>
       <c r="R44" s="2">
-        <v>2.4485486000000001E-2</v>
+        <v>2.4458997E-2</v>
       </c>
       <c r="S44" s="2">
-        <v>2.4475199999999999E-2</v>
+        <v>2.4535339E-2</v>
       </c>
       <c r="T44" s="2">
-        <v>2.4540763E-2</v>
+        <v>2.4587963000000001E-2</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="M45" s="2">
-        <v>4.9500071E-2</v>
+        <v>4.9610909000000002E-2</v>
       </c>
       <c r="N45" s="2">
-        <v>4.9320500000000003E-2</v>
+        <v>4.9344289999999999E-2</v>
       </c>
       <c r="O45" s="2">
-        <v>4.9038279999999997E-2</v>
+        <v>4.9302301999999999E-2</v>
       </c>
       <c r="P45" s="2">
-        <v>4.9267814E-2</v>
+        <v>4.9555529000000001E-2</v>
       </c>
       <c r="Q45" s="2">
-        <v>4.9049902999999999E-2</v>
+        <v>4.9348883000000003E-2</v>
       </c>
       <c r="R45" s="2">
-        <v>4.9062005999999998E-2</v>
+        <v>4.9216438000000001E-2</v>
       </c>
       <c r="S45" s="2">
-        <v>4.9283039000000001E-2</v>
+        <v>4.9488544000000002E-2</v>
       </c>
       <c r="T45" s="2">
-        <v>4.9481481000000001E-2</v>
+        <v>4.9386962999999999E-2</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
@@ -3369,28 +3369,28 @@
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
       <c r="M46" s="2">
-        <v>0.247341648</v>
+        <v>0.247525096</v>
       </c>
       <c r="N46" s="2">
-        <v>0.24609363100000001</v>
+        <v>0.24665647700000001</v>
       </c>
       <c r="O46" s="2">
-        <v>0.24456468200000001</v>
+        <v>0.245867804</v>
       </c>
       <c r="P46" s="2">
-        <v>0.24636517499999999</v>
+        <v>0.24723151300000001</v>
       </c>
       <c r="Q46" s="2">
-        <v>0.244711488</v>
+        <v>0.246422693</v>
       </c>
       <c r="R46" s="2">
-        <v>0.245086044</v>
+        <v>0.246523768</v>
       </c>
       <c r="S46" s="2">
-        <v>0.245740816</v>
+        <v>0.24664048899999999</v>
       </c>
       <c r="T46" s="2">
-        <v>0.24581067300000001</v>
+        <v>0.246864796</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
@@ -3422,28 +3422,28 @@
         <v>8</v>
       </c>
       <c r="M47" s="2">
-        <v>0.49444666500000001</v>
+        <v>0.49428844500000002</v>
       </c>
       <c r="N47" s="2">
-        <v>0.49110448400000001</v>
+        <v>0.491248727</v>
       </c>
       <c r="O47" s="2">
-        <v>0.48945605800000003</v>
+        <v>0.49277618499999998</v>
       </c>
       <c r="P47" s="2">
-        <v>0.49360141200000002</v>
+        <v>0.49547147800000002</v>
       </c>
       <c r="Q47" s="2">
-        <v>0.49054694199999999</v>
+        <v>0.49189487100000001</v>
       </c>
       <c r="R47" s="2">
-        <v>0.49154135599999998</v>
+        <v>0.49142217599999999</v>
       </c>
       <c r="S47" s="2">
-        <v>0.49097260799999998</v>
+        <v>0.492708117</v>
       </c>
       <c r="T47" s="2">
-        <v>0.49298122500000002</v>
+        <v>0.49235278399999999</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
@@ -3452,59 +3452,59 @@
       </c>
       <c r="B48" s="3">
         <f>M25*1000000</f>
-        <v>152.49993899999998</v>
+        <v>121.75425199999999</v>
       </c>
       <c r="C48" s="3">
         <f t="shared" ref="C48:I48" si="21">N25*1000000</f>
-        <v>140.64095700000001</v>
+        <v>120.79338199999999</v>
       </c>
       <c r="D48" s="3">
         <f t="shared" si="21"/>
-        <v>146.307153</v>
+        <v>122.003032</v>
       </c>
       <c r="E48" s="3">
         <f t="shared" si="21"/>
-        <v>143.88884300000001</v>
+        <v>126.82679499999999</v>
       </c>
       <c r="F48" s="3">
         <f t="shared" si="21"/>
-        <v>152.08304100000001</v>
+        <v>124.81863100000001</v>
       </c>
       <c r="G48" s="3">
         <f t="shared" si="21"/>
-        <v>156.41799800000001</v>
+        <v>126.072264</v>
       </c>
       <c r="H48" s="3">
         <f t="shared" si="21"/>
-        <v>138.09143299999999</v>
+        <v>121.47550299999999</v>
       </c>
       <c r="I48" s="3">
         <f t="shared" si="21"/>
-        <v>145.00779800000001</v>
+        <v>119.22544900000001</v>
       </c>
       <c r="M48" s="2">
-        <v>0.69277566700000004</v>
+        <v>0.69008028499999996</v>
       </c>
       <c r="N48" s="2">
-        <v>0.68740057899999996</v>
+        <v>0.687655091</v>
       </c>
       <c r="O48" s="2">
-        <v>0.684795916</v>
+        <v>0.68780779800000003</v>
       </c>
       <c r="P48" s="2">
-        <v>0.68962162699999996</v>
+        <v>0.69182115799999999</v>
       </c>
       <c r="Q48" s="2">
-        <v>0.68304491000000001</v>
+        <v>0.68727797300000004</v>
       </c>
       <c r="R48" s="2">
-        <v>0.68650931100000001</v>
+        <v>0.68697249900000001</v>
       </c>
       <c r="S48" s="2">
-        <v>0.68573868299999996</v>
+        <v>0.68911218600000002</v>
       </c>
       <c r="T48" s="2">
-        <v>0.68707990600000002</v>
+        <v>0.686764657</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.25">
@@ -3513,35 +3513,35 @@
       </c>
       <c r="B49" s="3">
         <f t="shared" ref="B49:B55" si="22">M26*1000000</f>
-        <v>481.40744899999999</v>
+        <v>476.82001600000001</v>
       </c>
       <c r="C49" s="3">
         <f t="shared" ref="C49:C55" si="23">N26*1000000</f>
-        <v>486.739125</v>
+        <v>476.15493500000002</v>
       </c>
       <c r="D49" s="3">
         <f t="shared" ref="D49:D55" si="24">O26*1000000</f>
-        <v>494.31267000000003</v>
+        <v>477.31155099999995</v>
       </c>
       <c r="E49" s="3">
         <f t="shared" ref="E49:E55" si="25">P26*1000000</f>
-        <v>487.818848</v>
+        <v>474.20134100000001</v>
       </c>
       <c r="F49" s="3">
         <f t="shared" ref="F49:F55" si="26">Q26*1000000</f>
-        <v>487.68019800000002</v>
+        <v>472.80560800000001</v>
       </c>
       <c r="G49" s="3">
         <f t="shared" ref="G49:G55" si="27">R26*1000000</f>
-        <v>487.26514800000001</v>
+        <v>476.71387400000003</v>
       </c>
       <c r="H49" s="3">
         <f t="shared" ref="H49:H55" si="28">S26*1000000</f>
-        <v>482.793723</v>
+        <v>475.71072399999997</v>
       </c>
       <c r="I49" s="3">
         <f t="shared" ref="I49:I55" si="29">T26*1000000</f>
-        <v>480.04451699999998</v>
+        <v>466.21434699999998</v>
       </c>
       <c r="M49" s="6">
         <v>9.9999997000000003E-5</v>
@@ -3574,35 +3574,35 @@
       </c>
       <c r="B50" s="3">
         <f t="shared" si="22"/>
-        <v>988.31742099999985</v>
+        <v>973.06759599999998</v>
       </c>
       <c r="C50" s="3">
         <f t="shared" si="23"/>
-        <v>971.54261299999996</v>
+        <v>960.03862599999991</v>
       </c>
       <c r="D50" s="3">
         <f t="shared" si="24"/>
-        <v>984.78992000000005</v>
+        <v>971.87486200000001</v>
       </c>
       <c r="E50" s="3">
         <f t="shared" si="25"/>
-        <v>978.97730300000012</v>
+        <v>977.9314280000001</v>
       </c>
       <c r="F50" s="3">
         <f t="shared" si="26"/>
-        <v>986.5829490000001</v>
+        <v>959.44979699999999</v>
       </c>
       <c r="G50" s="3">
         <f t="shared" si="27"/>
-        <v>991.40463900000009</v>
+        <v>975.22459700000002</v>
       </c>
       <c r="H50" s="3">
         <f t="shared" si="28"/>
-        <v>964.84430800000007</v>
+        <v>971.000001</v>
       </c>
       <c r="I50" s="3">
         <f t="shared" si="29"/>
-        <v>965.28546399999993</v>
+        <v>972.56735900000001</v>
       </c>
       <c r="M50" s="6">
         <v>5.0000002400000002E-4</v>
@@ -3635,35 +3635,35 @@
       </c>
       <c r="B51" s="3">
         <f t="shared" si="22"/>
-        <v>4945.0439999999999</v>
+        <v>4952.3890000000001</v>
       </c>
       <c r="C51" s="3">
         <f t="shared" si="23"/>
-        <v>4932.0550000000003</v>
+        <v>4936.3870000000006</v>
       </c>
       <c r="D51" s="3">
         <f t="shared" si="24"/>
-        <v>4963.7290000000003</v>
+        <v>4943.1659999999993</v>
       </c>
       <c r="E51" s="3">
         <f t="shared" si="25"/>
-        <v>4949.6030000000001</v>
+        <v>4930.0540000000001</v>
       </c>
       <c r="F51" s="3">
         <f t="shared" si="26"/>
-        <v>4967.8450000000003</v>
+        <v>4944.3910000000005</v>
       </c>
       <c r="G51" s="3">
         <f t="shared" si="27"/>
-        <v>4942.5449999999992</v>
+        <v>4951.1689999999999</v>
       </c>
       <c r="H51" s="3">
         <f t="shared" si="28"/>
-        <v>4945.2650000000003</v>
+        <v>4951.6289999999999</v>
       </c>
       <c r="I51" s="3">
         <f t="shared" si="29"/>
-        <v>4929.58</v>
+        <v>4938.54</v>
       </c>
       <c r="M51" s="6">
         <v>1E-3</v>
@@ -3696,35 +3696,35 @@
       </c>
       <c r="B52" s="3">
         <f t="shared" si="22"/>
-        <v>9915.2420000000002</v>
+        <v>9941.2860000000001</v>
       </c>
       <c r="C52" s="3">
         <f t="shared" si="23"/>
-        <v>9901.4270000000015</v>
+        <v>9897.7070000000003</v>
       </c>
       <c r="D52" s="3">
         <f t="shared" si="24"/>
-        <v>9950.9590000000007</v>
+        <v>9925.4009999999998</v>
       </c>
       <c r="E52" s="3">
         <f t="shared" si="25"/>
-        <v>9922.5609999999997</v>
+        <v>9910.5949999999993</v>
       </c>
       <c r="F52" s="3">
         <f t="shared" si="26"/>
-        <v>9939.3869999999988</v>
+        <v>9911.5540000000001</v>
       </c>
       <c r="G52" s="3">
         <f t="shared" si="27"/>
-        <v>9920.5419999999995</v>
+        <v>9951.482</v>
       </c>
       <c r="H52" s="3">
         <f t="shared" si="28"/>
-        <v>9896.2039999999997</v>
+        <v>9923.634</v>
       </c>
       <c r="I52" s="3">
         <f t="shared" si="29"/>
-        <v>9887.9760000000006</v>
+        <v>9939.17</v>
       </c>
       <c r="M52" s="6">
         <v>5.0000000000000001E-3</v>
@@ -3757,35 +3757,35 @@
       </c>
       <c r="B53" s="3">
         <f t="shared" si="22"/>
-        <v>49462.076000000001</v>
+        <v>49533.903999999995</v>
       </c>
       <c r="C53" s="3">
         <f t="shared" si="23"/>
-        <v>49399.659</v>
+        <v>49345.898999999998</v>
       </c>
       <c r="D53" s="3">
         <f t="shared" si="24"/>
-        <v>49613.386000000006</v>
+        <v>49606.13</v>
       </c>
       <c r="E53" s="3">
         <f t="shared" si="25"/>
-        <v>49500.73</v>
+        <v>49413.45</v>
       </c>
       <c r="F53" s="3">
         <f t="shared" si="26"/>
-        <v>49618.807000000001</v>
+        <v>49467.183999999994</v>
       </c>
       <c r="G53" s="3">
         <f t="shared" si="27"/>
-        <v>49608.263999999996</v>
+        <v>49669.548999999999</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" si="28"/>
-        <v>49478.78</v>
+        <v>49623.597000000002</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="29"/>
-        <v>49246.727999999996</v>
+        <v>49498.691999999995</v>
       </c>
       <c r="M53" s="6">
         <v>0.01</v>
@@ -3818,59 +3818,59 @@
       </c>
       <c r="B54" s="3">
         <f t="shared" si="22"/>
-        <v>98821.133000000002</v>
+        <v>98989.137000000002</v>
       </c>
       <c r="C54" s="3">
         <f t="shared" si="23"/>
-        <v>98632.857000000004</v>
+        <v>98584.622000000003</v>
       </c>
       <c r="D54" s="3">
         <f t="shared" si="24"/>
-        <v>99286.69</v>
+        <v>99155.97</v>
       </c>
       <c r="E54" s="3">
         <f t="shared" si="25"/>
-        <v>98927.698999999993</v>
+        <v>98913.892999999996</v>
       </c>
       <c r="F54" s="3">
         <f t="shared" si="26"/>
-        <v>98993.323999999993</v>
+        <v>98725.349000000002</v>
       </c>
       <c r="G54" s="3">
         <f t="shared" si="27"/>
-        <v>99263.869000000006</v>
+        <v>99280.453999999998</v>
       </c>
       <c r="H54" s="3">
         <f t="shared" si="28"/>
-        <v>98892.673999999999</v>
+        <v>99077.53</v>
       </c>
       <c r="I54" s="3">
         <f t="shared" si="29"/>
-        <v>98489.433999999994</v>
+        <v>98777.868000000002</v>
       </c>
       <c r="M54" s="6">
-        <v>4.9656693000000002E-2</v>
+        <v>4.9647706999999999E-2</v>
       </c>
       <c r="N54" s="6">
-        <v>4.9325801000000002E-2</v>
+        <v>4.9423195000000003E-2</v>
       </c>
       <c r="O54" s="6">
-        <v>4.9181014000000002E-2</v>
+        <v>4.9368504000000001E-2</v>
       </c>
       <c r="P54" s="6">
-        <v>4.9509554999999997E-2</v>
+        <v>4.9652311999999997E-2</v>
       </c>
       <c r="Q54" s="6">
-        <v>4.9130168000000002E-2</v>
+        <v>4.9482603E-2</v>
       </c>
       <c r="R54" s="6">
-        <v>4.9337458000000001E-2</v>
+        <v>4.9540794999999999E-2</v>
       </c>
       <c r="S54" s="6">
-        <v>4.9280349000000001E-2</v>
+        <v>4.9421663999999997E-2</v>
       </c>
       <c r="T54" s="6">
-        <v>4.9385492000000003E-2</v>
+        <v>4.9482651000000002E-2</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.25">
@@ -3879,85 +3879,85 @@
       </c>
       <c r="B55" s="3">
         <f t="shared" si="22"/>
-        <v>115692.213</v>
+        <v>114988.878</v>
       </c>
       <c r="C55" s="3">
         <f t="shared" si="23"/>
-        <v>113650.829</v>
+        <v>113413.326</v>
       </c>
       <c r="D55" s="3">
         <f t="shared" si="24"/>
-        <v>115137.629</v>
+        <v>115133.46400000001</v>
       </c>
       <c r="E55" s="3">
         <f t="shared" si="25"/>
-        <v>114977.136</v>
+        <v>114165.224</v>
       </c>
       <c r="F55" s="3">
         <f t="shared" si="26"/>
-        <v>112903.349</v>
+        <v>114818.394</v>
       </c>
       <c r="G55" s="3">
         <f t="shared" si="27"/>
-        <v>114548.489</v>
+        <v>115638.897</v>
       </c>
       <c r="H55" s="3">
         <f t="shared" si="28"/>
-        <v>113619.03700000001</v>
+        <v>114336.31199999999</v>
       </c>
       <c r="I55" s="3">
         <f t="shared" si="29"/>
-        <v>114151.902</v>
+        <v>114496.37299999999</v>
       </c>
       <c r="M55" s="6">
-        <v>9.9263579000000005E-2</v>
+        <v>9.9203572000000004E-2</v>
       </c>
       <c r="N55" s="6">
-        <v>9.8652034999999999E-2</v>
+        <v>9.8804719999999999E-2</v>
       </c>
       <c r="O55" s="6">
-        <v>9.8348170999999998E-2</v>
+        <v>9.8659708999999998E-2</v>
       </c>
       <c r="P55" s="6">
-        <v>9.8987310999999994E-2</v>
+        <v>9.9217295999999996E-2</v>
       </c>
       <c r="Q55" s="6">
-        <v>9.8288678000000004E-2</v>
+        <v>9.8895899999999995E-2</v>
       </c>
       <c r="R55" s="6">
-        <v>9.8649368000000001E-2</v>
+        <v>9.8979874999999995E-2</v>
       </c>
       <c r="S55" s="6">
-        <v>9.8553136E-2</v>
+        <v>9.8808460000000001E-2</v>
       </c>
       <c r="T55" s="6">
-        <v>9.8759234000000001E-2</v>
+        <v>9.8906754999999999E-2</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="M56" s="6">
-        <v>0.13853774999999999</v>
+        <v>0.13837470099999999</v>
       </c>
       <c r="N56" s="6">
-        <v>0.13773527699999999</v>
+        <v>0.13784571000000001</v>
       </c>
       <c r="O56" s="6">
-        <v>0.13729639399999999</v>
+        <v>0.13762928499999999</v>
       </c>
       <c r="P56" s="6">
-        <v>0.13817583</v>
+        <v>0.13839596500000001</v>
       </c>
       <c r="Q56" s="6">
-        <v>0.137259826</v>
+        <v>0.137978241</v>
       </c>
       <c r="R56" s="6">
-        <v>0.13769798</v>
+        <v>0.13807177500000001</v>
       </c>
       <c r="S56" s="6">
-        <v>0.137595087</v>
+        <v>0.13785977699999999</v>
       </c>
       <c r="T56" s="6">
-        <v>0.137883216</v>
+        <v>0.13798861200000001</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.25">
@@ -3973,28 +3973,28 @@
       <c r="H57" s="5"/>
       <c r="I57" s="5"/>
       <c r="M57" s="6">
-        <v>5.0662923600000001E-4</v>
+        <v>4.8846914400000002E-4</v>
       </c>
       <c r="N57" s="6">
-        <v>4.8821009100000001E-4</v>
+        <v>4.7766361999999999E-4</v>
       </c>
       <c r="O57" s="6">
-        <v>4.9999536699999998E-4</v>
+        <v>4.75040957E-4</v>
       </c>
       <c r="P57" s="6">
-        <v>4.7212955500000001E-4</v>
+        <v>4.6938305600000002E-4</v>
       </c>
       <c r="Q57" s="6">
-        <v>5.06367942E-4</v>
+        <v>4.7106656699999998E-4</v>
       </c>
       <c r="R57" s="6">
-        <v>4.8024085100000001E-4</v>
+        <v>4.7969026499999998E-4</v>
       </c>
       <c r="S57" s="6">
-        <v>4.8624887099999999E-4</v>
+        <v>4.9618503499999998E-4</v>
       </c>
       <c r="T57" s="6">
-        <v>4.8955710399999997E-4</v>
+        <v>4.78844915E-4</v>
       </c>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.25">
@@ -4026,28 +4026,28 @@
         <v>8</v>
       </c>
       <c r="M58" s="6">
-        <v>2.4437180000000001E-3</v>
+        <v>2.4208300000000001E-3</v>
       </c>
       <c r="N58" s="6">
-        <v>2.443794E-3</v>
+        <v>2.4243810000000002E-3</v>
       </c>
       <c r="O58" s="6">
-        <v>2.4389659999999999E-3</v>
+        <v>2.4276020000000001E-3</v>
       </c>
       <c r="P58" s="6">
-        <v>2.4397260000000001E-3</v>
+        <v>2.4272899999999999E-3</v>
       </c>
       <c r="Q58" s="6">
-        <v>2.4603030000000001E-3</v>
+        <v>2.4194809999999998E-3</v>
       </c>
       <c r="R58" s="6">
-        <v>2.4312040000000002E-3</v>
+        <v>2.4214639999999999E-3</v>
       </c>
       <c r="S58" s="6">
-        <v>2.4329690000000001E-3</v>
+        <v>2.4217840000000002E-3</v>
       </c>
       <c r="T58" s="6">
-        <v>2.4284749999999998E-3</v>
+        <v>2.4319839999999999E-3</v>
       </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.25">
@@ -4056,59 +4056,59 @@
       </c>
       <c r="B59" s="1">
         <f>B48-B37</f>
-        <v>152.49983900000299</v>
+        <v>121.75415200000299</v>
       </c>
       <c r="C59" s="1">
         <f t="shared" ref="C59:I59" si="30">C48-C37</f>
-        <v>140.64085700000302</v>
+        <v>120.79328200000299</v>
       </c>
       <c r="D59" s="1">
         <f t="shared" si="30"/>
-        <v>146.30705300000301</v>
+        <v>122.002932000003</v>
       </c>
       <c r="E59" s="1">
         <f t="shared" si="30"/>
-        <v>143.88874300000302</v>
+        <v>126.82669500000299</v>
       </c>
       <c r="F59" s="1">
         <f t="shared" si="30"/>
-        <v>152.08294100000302</v>
+        <v>124.81853100000301</v>
       </c>
       <c r="G59" s="1">
         <f t="shared" si="30"/>
-        <v>156.41789800000302</v>
+        <v>126.072164000003</v>
       </c>
       <c r="H59" s="1">
         <f t="shared" si="30"/>
-        <v>138.091333000003</v>
+        <v>121.47540300000298</v>
       </c>
       <c r="I59" s="1">
         <f t="shared" si="30"/>
-        <v>145.00769800000302</v>
+        <v>119.22534900000301</v>
       </c>
       <c r="M59" s="6">
-        <v>4.9529140000000001E-3</v>
+        <v>4.9532029999999998E-3</v>
       </c>
       <c r="N59" s="6">
-        <v>4.9534779999999999E-3</v>
+        <v>4.931342E-3</v>
       </c>
       <c r="O59" s="6">
-        <v>4.9638089999999996E-3</v>
+        <v>4.9600779999999997E-3</v>
       </c>
       <c r="P59" s="6">
-        <v>4.9541259999999997E-3</v>
+        <v>4.9342769999999999E-3</v>
       </c>
       <c r="Q59" s="6">
-        <v>4.9496239999999997E-3</v>
+        <v>4.939092E-3</v>
       </c>
       <c r="R59" s="6">
-        <v>4.948427E-3</v>
+        <v>4.9739939999999998E-3</v>
       </c>
       <c r="S59" s="6">
-        <v>4.9437420000000001E-3</v>
+        <v>4.9413210000000003E-3</v>
       </c>
       <c r="T59" s="6">
-        <v>4.9549950000000002E-3</v>
+        <v>4.947814E-3</v>
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.25">
@@ -4117,59 +4117,59 @@
       </c>
       <c r="B60" s="1">
         <f t="shared" ref="B60:I60" si="31">B49-B38</f>
-        <v>481.40694899997601</v>
+        <v>476.81951599997603</v>
       </c>
       <c r="C60" s="1">
         <f t="shared" si="31"/>
-        <v>486.73862499997603</v>
+        <v>476.15443499997605</v>
       </c>
       <c r="D60" s="1">
         <f t="shared" si="31"/>
-        <v>494.31216999997605</v>
+        <v>477.31105099997598</v>
       </c>
       <c r="E60" s="1">
         <f t="shared" si="31"/>
-        <v>487.81834799997603</v>
+        <v>474.20084099997604</v>
       </c>
       <c r="F60" s="1">
         <f t="shared" si="31"/>
-        <v>487.67969799997604</v>
+        <v>472.80510799997603</v>
       </c>
       <c r="G60" s="1">
         <f t="shared" si="31"/>
-        <v>487.26464799997603</v>
+        <v>476.71337399997606</v>
       </c>
       <c r="H60" s="1">
         <f t="shared" si="31"/>
-        <v>482.79322299997602</v>
+        <v>475.71022399997599</v>
       </c>
       <c r="I60" s="1">
         <f t="shared" si="31"/>
-        <v>480.04401699997601</v>
+        <v>466.213846999976</v>
       </c>
       <c r="M60" s="6">
-        <v>2.4944087E-2</v>
+        <v>2.4948146000000001E-2</v>
       </c>
       <c r="N60" s="6">
-        <v>2.4989687E-2</v>
+        <v>2.4928985000000001E-2</v>
       </c>
       <c r="O60" s="6">
-        <v>2.5008088000000001E-2</v>
+        <v>2.4940285999999999E-2</v>
       </c>
       <c r="P60" s="6">
-        <v>2.4973816999999999E-2</v>
+        <v>2.4846261000000001E-2</v>
       </c>
       <c r="Q60" s="6">
-        <v>2.5003435000000001E-2</v>
+        <v>2.4978118000000001E-2</v>
       </c>
       <c r="R60" s="6">
-        <v>2.4997152000000002E-2</v>
+        <v>2.4945729999999999E-2</v>
       </c>
       <c r="S60" s="6">
-        <v>2.4920688999999999E-2</v>
+        <v>2.4932466E-2</v>
       </c>
       <c r="T60" s="6">
-        <v>2.5012013E-2</v>
+        <v>2.4968183000000001E-2</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.25">
@@ -4178,59 +4178,59 @@
       </c>
       <c r="B61" s="1">
         <f t="shared" ref="B61:I61" si="32">B50-B39</f>
-        <v>988.31642099999988</v>
+        <v>973.066596</v>
       </c>
       <c r="C61" s="1">
         <f t="shared" si="32"/>
-        <v>971.54161299999998</v>
+        <v>960.03762599999993</v>
       </c>
       <c r="D61" s="1">
         <f t="shared" si="32"/>
-        <v>984.78892000000008</v>
+        <v>971.87386200000003</v>
       </c>
       <c r="E61" s="1">
         <f t="shared" si="32"/>
-        <v>978.97630300000014</v>
+        <v>977.93042800000012</v>
       </c>
       <c r="F61" s="1">
         <f t="shared" si="32"/>
-        <v>986.58194900000012</v>
+        <v>959.44879700000001</v>
       </c>
       <c r="G61" s="1">
         <f t="shared" si="32"/>
-        <v>991.40363900000011</v>
+        <v>975.22359700000004</v>
       </c>
       <c r="H61" s="1">
         <f t="shared" si="32"/>
-        <v>964.84330800000009</v>
+        <v>970.99900100000002</v>
       </c>
       <c r="I61" s="1">
         <f t="shared" si="32"/>
-        <v>965.28446399999996</v>
+        <v>972.56635900000003</v>
       </c>
       <c r="M61" s="6">
-        <v>4.9945913000000002E-2</v>
+        <v>4.9980719E-2</v>
       </c>
       <c r="N61" s="6">
-        <v>4.9900847999999998E-2</v>
+        <v>4.9968496000000001E-2</v>
       </c>
       <c r="O61" s="6">
-        <v>4.9965746999999998E-2</v>
+        <v>5.0003267999999997E-2</v>
       </c>
       <c r="P61" s="6">
-        <v>4.9951787999999997E-2</v>
+        <v>4.9803514E-2</v>
       </c>
       <c r="Q61" s="6">
-        <v>5.0054286000000003E-2</v>
+        <v>4.9950302000000002E-2</v>
       </c>
       <c r="R61" s="6">
-        <v>4.9915511000000003E-2</v>
+        <v>4.9947037999999999E-2</v>
       </c>
       <c r="S61" s="6">
-        <v>4.9948989999999999E-2</v>
+        <v>4.9917261999999997E-2</v>
       </c>
       <c r="T61" s="6">
-        <v>4.9986283999999999E-2</v>
+        <v>4.9917049999999998E-2</v>
       </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.25">
@@ -4239,59 +4239,59 @@
       </c>
       <c r="B62" s="1">
         <f t="shared" ref="B62:I62" si="33">B51-B40</f>
-        <v>4945.0389999999998</v>
+        <v>4952.384</v>
       </c>
       <c r="C62" s="1">
         <f t="shared" si="33"/>
-        <v>4932.05</v>
+        <v>4936.3820000000005</v>
       </c>
       <c r="D62" s="1">
         <f t="shared" si="33"/>
-        <v>4963.7240000000002</v>
+        <v>4943.1609999999991</v>
       </c>
       <c r="E62" s="1">
         <f t="shared" si="33"/>
-        <v>4949.598</v>
+        <v>4930.049</v>
       </c>
       <c r="F62" s="1">
         <f t="shared" si="33"/>
-        <v>4967.84</v>
+        <v>4944.3860000000004</v>
       </c>
       <c r="G62" s="1">
         <f t="shared" si="33"/>
-        <v>4942.5399999999991</v>
+        <v>4951.1639999999998</v>
       </c>
       <c r="H62" s="1">
         <f t="shared" si="33"/>
-        <v>4945.26</v>
+        <v>4951.6239999999998</v>
       </c>
       <c r="I62" s="1">
         <f t="shared" si="33"/>
-        <v>4929.5749999999998</v>
+        <v>4938.5349999999999</v>
       </c>
       <c r="M62" s="6">
-        <v>0.114046179</v>
+        <v>0.113534369</v>
       </c>
       <c r="N62" s="6">
-        <v>0.111845873</v>
+        <v>0.111855142</v>
       </c>
       <c r="O62" s="6">
-        <v>0.11342188</v>
+        <v>0.113344744</v>
       </c>
       <c r="P62" s="6">
-        <v>0.113214277</v>
+        <v>0.112271301</v>
       </c>
       <c r="Q62" s="6">
-        <v>0.11125861099999999</v>
+        <v>0.11298388199999999</v>
       </c>
       <c r="R62" s="6">
-        <v>0.112947218</v>
+        <v>0.11392086</v>
       </c>
       <c r="S62" s="6">
-        <v>0.111781903</v>
+        <v>0.112653427</v>
       </c>
       <c r="T62" s="6">
-        <v>0.11218500100000001</v>
+        <v>0.112591729</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.25">
@@ -4300,59 +4300,59 @@
       </c>
       <c r="B63" s="1">
         <f t="shared" ref="B63:I63" si="34">B52-B41</f>
-        <v>9915.232</v>
+        <v>9941.2759999999998</v>
       </c>
       <c r="C63" s="1">
         <f t="shared" si="34"/>
-        <v>9901.4170000000013</v>
+        <v>9897.6970000000001</v>
       </c>
       <c r="D63" s="1">
         <f t="shared" si="34"/>
-        <v>9950.9490000000005</v>
+        <v>9925.3909999999996</v>
       </c>
       <c r="E63" s="1">
         <f t="shared" si="34"/>
-        <v>9922.5509999999995</v>
+        <v>9910.5849999999991</v>
       </c>
       <c r="F63" s="1">
         <f t="shared" si="34"/>
-        <v>9939.3769999999986</v>
+        <v>9911.5439999999999</v>
       </c>
       <c r="G63" s="1">
         <f t="shared" si="34"/>
-        <v>9920.5319999999992</v>
+        <v>9951.4719999999998</v>
       </c>
       <c r="H63" s="1">
         <f t="shared" si="34"/>
-        <v>9896.1939999999995</v>
+        <v>9923.6239999999998</v>
       </c>
       <c r="I63" s="1">
         <f t="shared" si="34"/>
-        <v>9887.9660000000003</v>
+        <v>9939.16</v>
       </c>
       <c r="M63" s="6">
-        <v>0.11484119299999999</v>
+        <v>0.114707224</v>
       </c>
       <c r="N63" s="6">
-        <v>0.113151528</v>
+        <v>0.112819239</v>
       </c>
       <c r="O63" s="6">
-        <v>0.114190787</v>
+        <v>0.114495032</v>
       </c>
       <c r="P63" s="6">
-        <v>0.114100091</v>
+        <v>0.113293409</v>
       </c>
       <c r="Q63" s="6">
-        <v>0.111878715</v>
+        <v>0.11384040099999999</v>
       </c>
       <c r="R63" s="6">
-        <v>0.113634348</v>
+        <v>0.115043722</v>
       </c>
       <c r="S63" s="6">
-        <v>0.112822562</v>
+        <v>0.113871947</v>
       </c>
       <c r="T63" s="6">
-        <v>0.113111712</v>
+        <v>0.113781057</v>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.25">
@@ -4361,59 +4361,59 @@
       </c>
       <c r="B64" s="1">
         <f t="shared" ref="B64:I64" si="35">B53-B42</f>
-        <v>49462.026342814999</v>
+        <v>49533.854351055998</v>
       </c>
       <c r="C64" s="1">
         <f t="shared" si="35"/>
-        <v>49399.609677786</v>
+        <v>49345.849577847999</v>
       </c>
       <c r="D64" s="1">
         <f t="shared" si="35"/>
-        <v>49613.336819790005</v>
+        <v>49606.08063325</v>
       </c>
       <c r="E64" s="1">
         <f t="shared" si="35"/>
-        <v>49500.680489607003</v>
+        <v>49413.400349855998</v>
       </c>
       <c r="F64" s="1">
         <f t="shared" si="35"/>
-        <v>49618.757872891001</v>
+        <v>49467.134520798994</v>
       </c>
       <c r="G64" s="1">
         <f t="shared" si="35"/>
-        <v>49608.214666989996</v>
+        <v>49669.499458232</v>
       </c>
       <c r="H64" s="1">
         <f t="shared" si="35"/>
-        <v>49478.730719072999</v>
+        <v>49623.547579513004</v>
       </c>
       <c r="I64" s="1">
         <f t="shared" si="35"/>
-        <v>49246.678617581994</v>
+        <v>49498.642514919993</v>
       </c>
       <c r="M64" s="6">
-        <v>0.114772834</v>
+        <v>0.114523053</v>
       </c>
       <c r="N64" s="6">
-        <v>0.113101959</v>
+        <v>0.113101356</v>
       </c>
       <c r="O64" s="6">
-        <v>0.11430282899999999</v>
+        <v>0.11459907900000001</v>
       </c>
       <c r="P64" s="6">
-        <v>0.11426178400000001</v>
+        <v>0.11353451000000001</v>
       </c>
       <c r="Q64" s="6">
-        <v>0.112209797</v>
+        <v>0.113955691</v>
       </c>
       <c r="R64" s="6">
-        <v>0.113961756</v>
+        <v>0.114861675</v>
       </c>
       <c r="S64" s="6">
-        <v>0.113034829</v>
+        <v>0.11394001500000001</v>
       </c>
       <c r="T64" s="6">
-        <v>0.113282204</v>
+        <v>0.113695979</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -4422,35 +4422,35 @@
       </c>
       <c r="B65" s="1">
         <f t="shared" ref="B65:I65" si="36">B54-B43</f>
-        <v>98821.033742619999</v>
+        <v>98989.037802292005</v>
       </c>
       <c r="C65" s="1">
         <f t="shared" si="36"/>
-        <v>98632.758347399009</v>
+        <v>98584.523198752009</v>
       </c>
       <c r="D65" s="1">
         <f t="shared" si="36"/>
-        <v>99286.591647940004</v>
+        <v>99155.871344977</v>
       </c>
       <c r="E65" s="1">
         <f t="shared" si="36"/>
-        <v>98927.600009208996</v>
+        <v>98913.793786772003</v>
       </c>
       <c r="F65" s="1">
         <f t="shared" si="36"/>
-        <v>98993.22570861</v>
+        <v>98725.250101582002</v>
       </c>
       <c r="G65" s="1">
         <f t="shared" si="36"/>
-        <v>99263.770345849</v>
+        <v>99280.355019997995</v>
       </c>
       <c r="H65" s="1">
         <f t="shared" si="36"/>
-        <v>98892.575446900999</v>
+        <v>99077.431198029997</v>
       </c>
       <c r="I65" s="1">
         <f t="shared" si="36"/>
-        <v>98489.335243388996</v>
+        <v>98777.769098043005</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -4459,35 +4459,35 @@
       </c>
       <c r="B66" s="1">
         <f t="shared" ref="B66:I66" si="37">B55-B44</f>
-        <v>115692.074468256</v>
+        <v>114988.73963262999</v>
       </c>
       <c r="C66" s="1">
         <f t="shared" si="37"/>
-        <v>113650.691278834</v>
+        <v>113413.188152442</v>
       </c>
       <c r="D66" s="1">
         <f t="shared" si="37"/>
-        <v>115137.491726972</v>
+        <v>115133.32637174301</v>
       </c>
       <c r="E66" s="1">
         <f t="shared" si="37"/>
-        <v>114976.997849412</v>
+        <v>114165.0855973</v>
       </c>
       <c r="F66" s="1">
         <f t="shared" si="37"/>
-        <v>112903.211745181</v>
+        <v>114818.256021953</v>
       </c>
       <c r="G66" s="1">
         <f t="shared" si="37"/>
-        <v>114548.351300724</v>
+        <v>115638.75893424499</v>
       </c>
       <c r="H66" s="1">
         <f t="shared" si="37"/>
-        <v>113618.899415552</v>
+        <v>114336.174139061</v>
       </c>
       <c r="I66" s="1">
         <f t="shared" si="37"/>
-        <v>114151.76411994301</v>
+        <v>114496.23501102999</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -4723,35 +4723,35 @@
       </c>
       <c r="B75" s="3">
         <f t="shared" si="39"/>
-        <v>4.9655095000000003E-2</v>
+        <v>4.9650811000000003E-2</v>
       </c>
       <c r="C75" s="3">
         <f t="shared" si="40"/>
-        <v>4.9324519999999997E-2</v>
+        <v>4.9422219000000003E-2</v>
       </c>
       <c r="D75" s="3">
         <f t="shared" si="41"/>
-        <v>4.9180791000000001E-2</v>
+        <v>4.9367290000000001E-2</v>
       </c>
       <c r="E75" s="3">
         <f t="shared" si="42"/>
-        <v>4.9508496999999999E-2</v>
+        <v>4.9646094000000002E-2</v>
       </c>
       <c r="F75" s="3">
         <f t="shared" si="43"/>
-        <v>4.9131345E-2</v>
+        <v>4.9480746999999999E-2</v>
       </c>
       <c r="G75" s="3">
         <f t="shared" si="44"/>
-        <v>4.9340144000000002E-2</v>
+        <v>4.9538441000000003E-2</v>
       </c>
       <c r="H75" s="3">
         <f t="shared" si="45"/>
-        <v>4.9281432999999999E-2</v>
+        <v>4.9419998999999999E-2</v>
       </c>
       <c r="I75" s="3">
         <f t="shared" si="46"/>
-        <v>4.9382750000000003E-2</v>
+        <v>4.9482878000000001E-2</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -4760,35 +4760,35 @@
       </c>
       <c r="B76" s="3">
         <f t="shared" si="39"/>
-        <v>9.9262929999999999E-2</v>
+        <v>9.9202491000000004E-2</v>
       </c>
       <c r="C76" s="3">
         <f t="shared" si="40"/>
-        <v>9.8648741999999998E-2</v>
+        <v>9.8805428000000001E-2</v>
       </c>
       <c r="D76" s="3">
         <f t="shared" si="41"/>
-        <v>9.8343431999999995E-2</v>
+        <v>9.8655857E-2</v>
       </c>
       <c r="E76" s="3">
         <f t="shared" si="42"/>
-        <v>9.8990038000000002E-2</v>
+        <v>9.9210665000000003E-2</v>
       </c>
       <c r="F76" s="3">
         <f t="shared" si="43"/>
-        <v>9.8295055000000006E-2</v>
+        <v>9.8896242999999995E-2</v>
       </c>
       <c r="G76" s="3">
         <f t="shared" si="44"/>
-        <v>9.8657139000000005E-2</v>
+        <v>9.8978109999999994E-2</v>
       </c>
       <c r="H76" s="3">
         <f t="shared" si="45"/>
-        <v>9.8554007999999999E-2</v>
+        <v>9.8800674000000005E-2</v>
       </c>
       <c r="I76" s="3">
         <f t="shared" si="46"/>
-        <v>9.8760411000000006E-2</v>
+        <v>9.8902008999999999E-2</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -4797,35 +4797,35 @@
       </c>
       <c r="B77" s="3">
         <f t="shared" si="39"/>
-        <v>0.13853786900000001</v>
+        <v>0.138369307</v>
       </c>
       <c r="C77" s="3">
         <f t="shared" si="40"/>
-        <v>0.13773238700000001</v>
+        <v>0.137844458</v>
       </c>
       <c r="D77" s="3">
         <f t="shared" si="41"/>
-        <v>0.13728112000000001</v>
+        <v>0.137627363</v>
       </c>
       <c r="E77" s="3">
         <f t="shared" si="42"/>
-        <v>0.138173938</v>
+        <v>0.138406157</v>
       </c>
       <c r="F77" s="3">
         <f t="shared" si="43"/>
-        <v>0.13726683000000001</v>
+        <v>0.137964159</v>
       </c>
       <c r="G77" s="3">
         <f t="shared" si="44"/>
-        <v>0.137702301</v>
+        <v>0.13806495099999999</v>
       </c>
       <c r="H77" s="3">
         <f t="shared" si="45"/>
-        <v>0.137587458</v>
+        <v>0.13785430800000001</v>
       </c>
       <c r="I77" s="3">
         <f t="shared" si="46"/>
-        <v>0.13789103899999999</v>
+        <v>0.13798032700000001</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -4876,35 +4876,35 @@
       </c>
       <c r="B81" s="3">
         <f>(M41/5)*1000000</f>
-        <v>63.6066194</v>
+        <v>84.944092600000005</v>
       </c>
       <c r="C81" s="3">
         <f t="shared" ref="C81:I81" si="47">(N41/5)*1000000</f>
-        <v>61.542465200000009</v>
+        <v>84.179989000000006</v>
       </c>
       <c r="D81" s="3">
         <f t="shared" si="47"/>
-        <v>69.576199200000005</v>
+        <v>78.448373799999985</v>
       </c>
       <c r="E81" s="3">
         <f t="shared" si="47"/>
-        <v>72.445126799999997</v>
+        <v>81.473769399999995</v>
       </c>
       <c r="F81" s="3">
         <f t="shared" si="47"/>
-        <v>67.384424600000003</v>
+        <v>86.981442200000004</v>
       </c>
       <c r="G81" s="3">
         <f t="shared" si="47"/>
-        <v>63.153070999999997</v>
+        <v>81.61892180000001</v>
       </c>
       <c r="H81" s="3">
         <f t="shared" si="47"/>
-        <v>69.834431600000002</v>
+        <v>82.382588799999994</v>
       </c>
       <c r="I81" s="3">
         <f t="shared" si="47"/>
-        <v>66.738971599999999</v>
+        <v>87.130081399999995</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -4913,35 +4913,35 @@
       </c>
       <c r="B82" s="3">
         <f t="shared" ref="B82:B88" si="48">(M42/5)*1000000</f>
-        <v>442.17740000000003</v>
+        <v>434.21719999999999</v>
       </c>
       <c r="C82" s="3">
         <f t="shared" ref="C82:C88" si="49">(N42/5)*1000000</f>
-        <v>437.7824</v>
+        <v>429.00799999999998</v>
       </c>
       <c r="D82" s="3">
         <f t="shared" ref="D82:D88" si="50">(O42/5)*1000000</f>
-        <v>439.74580000000003</v>
+        <v>432.64699999999999</v>
       </c>
       <c r="E82" s="3">
         <f t="shared" ref="E82:E88" si="51">(P42/5)*1000000</f>
-        <v>438.83600000000001</v>
+        <v>434.4228</v>
       </c>
       <c r="F82" s="3">
         <f t="shared" ref="F82:F88" si="52">(Q42/5)*1000000</f>
-        <v>439.63359999999994</v>
+        <v>430.452</v>
       </c>
       <c r="G82" s="3">
         <f t="shared" ref="G82:G88" si="53">(R42/5)*1000000</f>
-        <v>434.89879999999999</v>
+        <v>430.94819999999999</v>
       </c>
       <c r="H82" s="3">
         <f t="shared" ref="H82:H88" si="54">(S42/5)*1000000</f>
-        <v>435.36800000000005</v>
+        <v>431.35880000000003</v>
       </c>
       <c r="I82" s="3">
         <f t="shared" ref="I82:I88" si="55">(T42/5)*1000000</f>
-        <v>440.03899999999999</v>
+        <v>433.75059999999996</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -4950,35 +4950,35 @@
       </c>
       <c r="B83" s="3">
         <f t="shared" si="48"/>
-        <v>943.49779999999998</v>
+        <v>937.22119999999995</v>
       </c>
       <c r="C83" s="3">
         <f t="shared" si="49"/>
-        <v>940.04099999999994</v>
+        <v>937.7808</v>
       </c>
       <c r="D83" s="3">
         <f t="shared" si="50"/>
-        <v>937.97659999999996</v>
+        <v>935.1386</v>
       </c>
       <c r="E83" s="3">
         <f t="shared" si="51"/>
-        <v>939.25059999999996</v>
+        <v>940.76400000000001</v>
       </c>
       <c r="F83" s="3">
         <f t="shared" si="52"/>
-        <v>934.0598</v>
+        <v>936.51340000000005</v>
       </c>
       <c r="G83" s="3">
         <f t="shared" si="53"/>
-        <v>935.45920000000001</v>
+        <v>934.05280000000005</v>
       </c>
       <c r="H83" s="3">
         <f t="shared" si="54"/>
-        <v>936.93160000000012</v>
+        <v>936.75840000000005</v>
       </c>
       <c r="I83" s="3">
         <f t="shared" si="55"/>
-        <v>940.88459999999998</v>
+        <v>936.1318</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -4987,35 +4987,35 @@
       </c>
       <c r="B84" s="3">
         <f t="shared" si="48"/>
-        <v>4935.5801999999994</v>
+        <v>4936.2450000000008</v>
       </c>
       <c r="C84" s="3">
         <f t="shared" si="49"/>
-        <v>4903.442</v>
+        <v>4900.5411999999997</v>
       </c>
       <c r="D84" s="3">
         <f t="shared" si="50"/>
-        <v>4896.4495999999999</v>
+        <v>4890.5457999999999</v>
       </c>
       <c r="E84" s="3">
         <f t="shared" si="51"/>
-        <v>4907.5349999999989</v>
+        <v>4934.6337999999996</v>
       </c>
       <c r="F84" s="3">
         <f t="shared" si="52"/>
-        <v>4896.3946000000005</v>
+        <v>4906.5362000000005</v>
       </c>
       <c r="G84" s="3">
         <f t="shared" si="53"/>
-        <v>4897.0972000000002</v>
+        <v>4891.7993999999999</v>
       </c>
       <c r="H84" s="3">
         <f t="shared" si="54"/>
-        <v>4895.04</v>
+        <v>4907.0677999999998</v>
       </c>
       <c r="I84" s="3">
         <f t="shared" si="55"/>
-        <v>4908.1526000000003</v>
+        <v>4917.5925999999999</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -5024,35 +5024,35 @@
       </c>
       <c r="B85" s="3">
         <f t="shared" si="48"/>
-        <v>9900.0141999999996</v>
+        <v>9922.1818000000003</v>
       </c>
       <c r="C85" s="3">
         <f t="shared" si="49"/>
-        <v>9864.1</v>
+        <v>9868.8580000000002</v>
       </c>
       <c r="D85" s="3">
         <f t="shared" si="50"/>
-        <v>9807.655999999999</v>
+        <v>9860.4603999999999</v>
       </c>
       <c r="E85" s="3">
         <f t="shared" si="51"/>
-        <v>9853.5627999999997</v>
+        <v>9911.1057999999994</v>
       </c>
       <c r="F85" s="3">
         <f t="shared" si="52"/>
-        <v>9809.9806000000008</v>
+        <v>9869.7766000000011</v>
       </c>
       <c r="G85" s="3">
         <f t="shared" si="53"/>
-        <v>9812.4011999999984</v>
+        <v>9843.2875999999997</v>
       </c>
       <c r="H85" s="3">
         <f t="shared" si="54"/>
-        <v>9856.6077999999998</v>
+        <v>9897.7088000000003</v>
       </c>
       <c r="I85" s="3">
         <f t="shared" si="55"/>
-        <v>9896.2962000000007</v>
+        <v>9877.3925999999992</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -5061,35 +5061,35 @@
       </c>
       <c r="B86" s="3">
         <f t="shared" si="48"/>
-        <v>49468.329599999997</v>
+        <v>49505.019200000002</v>
       </c>
       <c r="C86" s="3">
         <f t="shared" si="49"/>
-        <v>49218.726199999997</v>
+        <v>49331.295400000003</v>
       </c>
       <c r="D86" s="3">
         <f t="shared" si="50"/>
-        <v>48912.936400000006</v>
+        <v>49173.560799999999</v>
       </c>
       <c r="E86" s="3">
         <f t="shared" si="51"/>
-        <v>49273.034999999996</v>
+        <v>49446.302600000003</v>
       </c>
       <c r="F86" s="3">
         <f t="shared" si="52"/>
-        <v>48942.297600000005</v>
+        <v>49284.5386</v>
       </c>
       <c r="G86" s="3">
         <f t="shared" si="53"/>
-        <v>49017.2088</v>
+        <v>49304.753600000004</v>
       </c>
       <c r="H86" s="3">
         <f t="shared" si="54"/>
-        <v>49148.163199999995</v>
+        <v>49328.097799999996</v>
       </c>
       <c r="I86" s="3">
         <f t="shared" si="55"/>
-        <v>49162.134600000005</v>
+        <v>49372.959199999998</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -5098,35 +5098,35 @@
       </c>
       <c r="B87" s="3">
         <f t="shared" si="48"/>
-        <v>98889.332999999999</v>
+        <v>98857.688999999998</v>
       </c>
       <c r="C87" s="3">
         <f t="shared" si="49"/>
-        <v>98220.896800000002</v>
+        <v>98249.7454</v>
       </c>
       <c r="D87" s="3">
         <f t="shared" si="50"/>
-        <v>97891.211599999995</v>
+        <v>98555.236999999994</v>
       </c>
       <c r="E87" s="3">
         <f t="shared" si="51"/>
-        <v>98720.282399999996</v>
+        <v>99094.295600000012</v>
       </c>
       <c r="F87" s="3">
         <f t="shared" si="52"/>
-        <v>98109.388399999996</v>
+        <v>98378.974199999997</v>
       </c>
       <c r="G87" s="3">
         <f t="shared" si="53"/>
-        <v>98308.271199999988</v>
+        <v>98284.435199999993</v>
       </c>
       <c r="H87" s="3">
         <f t="shared" si="54"/>
-        <v>98194.521600000007</v>
+        <v>98541.623399999997</v>
       </c>
       <c r="I87" s="3">
         <f t="shared" si="55"/>
-        <v>98596.244999999995</v>
+        <v>98470.556799999991</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,35 +5135,35 @@
       </c>
       <c r="B88" s="3">
         <f t="shared" si="48"/>
-        <v>138555.13339999999</v>
+        <v>138016.057</v>
       </c>
       <c r="C88" s="3">
         <f t="shared" si="49"/>
-        <v>137480.1158</v>
+        <v>137531.01819999999</v>
       </c>
       <c r="D88" s="3">
         <f t="shared" si="50"/>
-        <v>136959.1832</v>
+        <v>137561.55960000001</v>
       </c>
       <c r="E88" s="3">
         <f t="shared" si="51"/>
-        <v>137924.3254</v>
+        <v>138364.2316</v>
       </c>
       <c r="F88" s="3">
         <f t="shared" si="52"/>
-        <v>136608.98199999999</v>
+        <v>137455.59460000001</v>
       </c>
       <c r="G88" s="3">
         <f t="shared" si="53"/>
-        <v>137301.8622</v>
+        <v>137394.49980000002</v>
       </c>
       <c r="H88" s="3">
         <f t="shared" si="54"/>
-        <v>137147.73659999997</v>
+        <v>137822.43720000001</v>
       </c>
       <c r="I88" s="3">
         <f t="shared" si="55"/>
-        <v>137415.98120000001</v>
+        <v>137352.9314</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -5214,35 +5214,35 @@
       </c>
       <c r="B92" s="1">
         <f>B81-B70</f>
-        <v>63.606519400003002</v>
+        <v>84.943992600003</v>
       </c>
       <c r="C92" s="1">
         <f t="shared" ref="C92:I92" si="56">C81-C70</f>
-        <v>61.542365200003012</v>
+        <v>84.179889000003001</v>
       </c>
       <c r="D92" s="1">
         <f t="shared" si="56"/>
-        <v>69.576099200003</v>
+        <v>78.44827380000298</v>
       </c>
       <c r="E92" s="1">
         <f t="shared" si="56"/>
-        <v>72.445026800002992</v>
+        <v>81.47366940000299</v>
       </c>
       <c r="F92" s="1">
         <f t="shared" si="56"/>
-        <v>67.384324600002998</v>
+        <v>86.981342200002999</v>
       </c>
       <c r="G92" s="1">
         <f t="shared" si="56"/>
-        <v>63.152971000002999</v>
+        <v>81.618821800003005</v>
       </c>
       <c r="H92" s="1">
         <f t="shared" si="56"/>
-        <v>69.834331600002997</v>
+        <v>82.382488800002989</v>
       </c>
       <c r="I92" s="1">
         <f t="shared" si="56"/>
-        <v>66.738871600002994</v>
+        <v>87.12998140000299</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,35 +5251,35 @@
       </c>
       <c r="B93" s="1">
         <f t="shared" ref="B93:I93" si="57">B82-B71</f>
-        <v>442.17689999997606</v>
+        <v>434.21669999997602</v>
       </c>
       <c r="C93" s="1">
         <f t="shared" si="57"/>
-        <v>437.78189999997602</v>
+        <v>429.00749999997601</v>
       </c>
       <c r="D93" s="1">
         <f t="shared" si="57"/>
-        <v>439.74529999997606</v>
+        <v>432.64649999997602</v>
       </c>
       <c r="E93" s="1">
         <f t="shared" si="57"/>
-        <v>438.83549999997604</v>
+        <v>434.42229999997602</v>
       </c>
       <c r="F93" s="1">
         <f t="shared" si="57"/>
-        <v>439.63309999997597</v>
+        <v>430.45149999997602</v>
       </c>
       <c r="G93" s="1">
         <f t="shared" si="57"/>
-        <v>434.89829999997602</v>
+        <v>430.94769999997601</v>
       </c>
       <c r="H93" s="1">
         <f t="shared" si="57"/>
-        <v>435.36749999997608</v>
+        <v>431.35829999997605</v>
       </c>
       <c r="I93" s="1">
         <f t="shared" si="57"/>
-        <v>440.03849999997601</v>
+        <v>433.75009999997599</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -5288,35 +5288,35 @@
       </c>
       <c r="B94" s="1">
         <f t="shared" ref="B94:I94" si="58">B83-B72</f>
-        <v>943.49680000000001</v>
+        <v>937.22019999999998</v>
       </c>
       <c r="C94" s="1">
         <f t="shared" si="58"/>
-        <v>940.04</v>
+        <v>937.77980000000002</v>
       </c>
       <c r="D94" s="1">
         <f t="shared" si="58"/>
-        <v>937.97559999999999</v>
+        <v>935.13760000000002</v>
       </c>
       <c r="E94" s="1">
         <f t="shared" si="58"/>
-        <v>939.24959999999999</v>
+        <v>940.76300000000003</v>
       </c>
       <c r="F94" s="1">
         <f t="shared" si="58"/>
-        <v>934.05880000000002</v>
+        <v>936.51240000000007</v>
       </c>
       <c r="G94" s="1">
         <f t="shared" si="58"/>
-        <v>935.45820000000003</v>
+        <v>934.05180000000007</v>
       </c>
       <c r="H94" s="1">
         <f t="shared" si="58"/>
-        <v>936.93060000000014</v>
+        <v>936.75740000000008</v>
       </c>
       <c r="I94" s="1">
         <f t="shared" si="58"/>
-        <v>940.8836</v>
+        <v>936.13080000000002</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -5325,35 +5325,35 @@
       </c>
       <c r="B95" s="1">
         <f t="shared" ref="B95:I95" si="59">B84-B73</f>
-        <v>4935.5751999999993</v>
+        <v>4936.2400000000007</v>
       </c>
       <c r="C95" s="1">
         <f t="shared" si="59"/>
-        <v>4903.4369999999999</v>
+        <v>4900.5361999999996</v>
       </c>
       <c r="D95" s="1">
         <f t="shared" si="59"/>
-        <v>4896.4445999999998</v>
+        <v>4890.5407999999998</v>
       </c>
       <c r="E95" s="1">
         <f t="shared" si="59"/>
-        <v>4907.5299999999988</v>
+        <v>4934.6287999999995</v>
       </c>
       <c r="F95" s="1">
         <f t="shared" si="59"/>
-        <v>4896.3896000000004</v>
+        <v>4906.5312000000004</v>
       </c>
       <c r="G95" s="1">
         <f t="shared" si="59"/>
-        <v>4897.0922</v>
+        <v>4891.7943999999998</v>
       </c>
       <c r="H95" s="1">
         <f t="shared" si="59"/>
-        <v>4895.0349999999999</v>
+        <v>4907.0627999999997</v>
       </c>
       <c r="I95" s="1">
         <f t="shared" si="59"/>
-        <v>4908.1476000000002</v>
+        <v>4917.5875999999998</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -5362,35 +5362,35 @@
       </c>
       <c r="B96" s="1">
         <f t="shared" ref="B96:I96" si="60">B85-B74</f>
-        <v>9900.0041999999994</v>
+        <v>9922.1718000000001</v>
       </c>
       <c r="C96" s="1">
         <f t="shared" si="60"/>
-        <v>9864.09</v>
+        <v>9868.848</v>
       </c>
       <c r="D96" s="1">
         <f t="shared" si="60"/>
-        <v>9807.6459999999988</v>
+        <v>9860.4503999999997</v>
       </c>
       <c r="E96" s="1">
         <f t="shared" si="60"/>
-        <v>9853.5527999999995</v>
+        <v>9911.0957999999991</v>
       </c>
       <c r="F96" s="1">
         <f t="shared" si="60"/>
-        <v>9809.9706000000006</v>
+        <v>9869.7666000000008</v>
       </c>
       <c r="G96" s="1">
         <f t="shared" si="60"/>
-        <v>9812.3911999999982</v>
+        <v>9843.2775999999994</v>
       </c>
       <c r="H96" s="1">
         <f t="shared" si="60"/>
-        <v>9856.5977999999996</v>
+        <v>9897.6988000000001</v>
       </c>
       <c r="I96" s="1">
         <f t="shared" si="60"/>
-        <v>9896.2862000000005</v>
+        <v>9877.382599999999</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -5399,35 +5399,35 @@
       </c>
       <c r="B97" s="1">
         <f t="shared" ref="B97:I97" si="61">B86-B75</f>
-        <v>49468.279944905</v>
+        <v>49504.969549189002</v>
       </c>
       <c r="C97" s="1">
         <f t="shared" si="61"/>
-        <v>49218.67687548</v>
+        <v>49331.245977781</v>
       </c>
       <c r="D97" s="1">
         <f t="shared" si="61"/>
-        <v>48912.887219209006</v>
+        <v>49173.511432710002</v>
       </c>
       <c r="E97" s="1">
         <f t="shared" si="61"/>
-        <v>49272.985491502994</v>
+        <v>49446.252953906005</v>
       </c>
       <c r="F97" s="1">
         <f t="shared" si="61"/>
-        <v>48942.248468655009</v>
+        <v>49284.489119252998</v>
       </c>
       <c r="G97" s="1">
         <f t="shared" si="61"/>
-        <v>49017.159459855997</v>
+        <v>49304.704061559001</v>
       </c>
       <c r="H97" s="1">
         <f t="shared" si="61"/>
-        <v>49148.113918566996</v>
+        <v>49328.048380000997</v>
       </c>
       <c r="I97" s="1">
         <f t="shared" si="61"/>
-        <v>49162.085217250002</v>
+        <v>49372.909717121998</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -5436,35 +5436,35 @@
       </c>
       <c r="B98" s="1">
         <f t="shared" ref="B98:I98" si="62">B87-B76</f>
-        <v>98889.233737069997</v>
+        <v>98857.589797509005</v>
       </c>
       <c r="C98" s="1">
         <f t="shared" si="62"/>
-        <v>98220.798151258001</v>
+        <v>98249.646594571997</v>
       </c>
       <c r="D98" s="1">
         <f t="shared" si="62"/>
-        <v>97891.113256568002</v>
+        <v>98555.138344142993</v>
       </c>
       <c r="E98" s="1">
         <f t="shared" si="62"/>
-        <v>98720.183409962003</v>
+        <v>99094.196389335018</v>
       </c>
       <c r="F98" s="1">
         <f t="shared" si="62"/>
-        <v>98109.290104945001</v>
+        <v>98378.875303756999</v>
       </c>
       <c r="G98" s="1">
         <f t="shared" si="62"/>
-        <v>98308.172542860993</v>
+        <v>98284.336221889986</v>
       </c>
       <c r="H98" s="1">
         <f t="shared" si="62"/>
-        <v>98194.423045992007</v>
+        <v>98541.524599326003</v>
       </c>
       <c r="I98" s="1">
         <f t="shared" si="62"/>
-        <v>98596.146239588998</v>
+        <v>98470.457897990986</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
@@ -5473,35 +5473,35 @@
       </c>
       <c r="B99" s="1">
         <f t="shared" ref="B99:I99" si="63">B88-B77</f>
-        <v>138554.99486213099</v>
+        <v>138015.91863069299</v>
       </c>
       <c r="C99" s="1">
         <f t="shared" si="63"/>
-        <v>137479.978067613</v>
+        <v>137530.880355542</v>
       </c>
       <c r="D99" s="1">
         <f t="shared" si="63"/>
-        <v>136959.04591888</v>
+        <v>137561.42197263701</v>
       </c>
       <c r="E99" s="1">
         <f t="shared" si="63"/>
-        <v>137924.187226062</v>
+        <v>138364.093193843</v>
       </c>
       <c r="F99" s="1">
         <f t="shared" si="63"/>
-        <v>136608.84473317</v>
+        <v>137455.45663584102</v>
       </c>
       <c r="G99" s="1">
         <f t="shared" si="63"/>
-        <v>137301.724497699</v>
+        <v>137394.36173504902</v>
       </c>
       <c r="H99" s="1">
         <f t="shared" si="63"/>
-        <v>137147.59901254196</v>
+        <v>137822.29934569201</v>
       </c>
       <c r="I99" s="1">
         <f t="shared" si="63"/>
-        <v>137415.84330896102</v>
+        <v>137352.79341967299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>